<commit_message>
Tailor the system to the Nuclear and Radiological Regulatory Commission
- Default organisation name in the app header and reports
- Logo upload suggests report colours from the logo
- Suggested regulatory categories and an inspection event type
- Regulatory-themed sample data and refreshed sample reports

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vq5DRv9yx8RnT5NY8AHtK
</commit_message>
<xml_diff>
--- a/samples/5-ملف-Excel.xlsx
+++ b/samples/5-ملف-Excel.xlsx
@@ -18,29 +18,29 @@
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="O4" authorId="0">
+    <comment ref="K4" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/21 – فتح الموضوع
+          <t xml:space="preserve">2026/08/22 – فتح الموضوع
 تسجيل الموضوع
-2026/09/23 – مراسلة
-مراسلة الجهة لطلب وثائق الربط</t>
+2026/08/27 – اجتماع
+ورشة عمل داخلية لمراجعة المسودة الأولى</t>
         </r>
       </text>
     </comment>
-    <comment ref="P4" authorId="0">
+    <comment ref="M4" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/10/02 – اجتماع
-اجتماع فني مع فريق الجهة</t>
+          <t xml:space="preserve">2026/09/11 – إجراء
+طرح المسودة لأخذ مرئيات الجهات ذات العلاقة</t>
         </r>
       </text>
     </comment>
     <comment ref="Q4" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/10/09 – تحديث
-استلام بيئة الاختبار</t>
+          <t xml:space="preserve">2026/10/07 – تحديث
+استلام 12 مرئية من الجهات</t>
         </r>
       </text>
     </comment>
@@ -48,7 +48,7 @@
       <text>
         <r>
           <t xml:space="preserve">2026/09/01 – فتح الموضوع
-تسجيل الموضوع: انتهاء عقد الصيانة الحالي ويلزم الطرح والترسية قبل نهاية الربع لضمان استمرارية الخدمة.</t>
+تسجيل الموضوع: طلب ترخيص جديد لاستخدام مصادر مشعة في العلاج الإشعاعي، ويتطلب استيفاء متطلبات الدروع والتقييم الإشعاعي قبل إصدار الترخيص.</t>
         </r>
       </text>
     </comment>
@@ -56,23 +56,23 @@
       <text>
         <r>
           <t xml:space="preserve">2026/09/06 – مراسلة (أحمد العتيبي)
-إرسال خطاب لإدارة المشتريات بطلب طرح المنافسة</t>
+إرسال خطاب للجهة بطلب استيفاء متطلبات الدروع وخطة الوقاية الإشعاعية</t>
         </r>
       </text>
     </comment>
     <comment ref="N5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/13 – اجتماع (لجنة العقود)
-اجتماع مع المشتريات لمراجعة كراسة الشروط واعتماد نطاق العمل</t>
+          <t xml:space="preserve">2026/09/15 – تفتيش / زيارة ميدانية (فريق التفتيش)
+زيارة ميدانية للتحقق من غرفة العلاج وأنظمة الدروع؛ رُصدت 3 ملاحظات</t>
         </r>
       </text>
     </comment>
     <comment ref="P5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/26 – إجراء (إدارة المشتريات)
-طرح المنافسة واستقبال ثلاثة عروض من المقاولين المؤهلين</t>
+          <t xml:space="preserve">2026/09/26 – اجتماع (إدارة التراخيص)
+اجتماع مع الجهة لمناقشة خطة معالجة الملاحظات وجدولها الزمني</t>
         </r>
       </text>
     </comment>
@@ -80,7 +80,7 @@
       <text>
         <r>
           <t xml:space="preserve">2026/10/05 – متابعة (أحمد العتيبي)
-متابعة التقييم الفني للعروض – بانتظار اجتماع لجنة الفحص</t>
+متابعة تنفيذ تعديلات الدروع – بانتظار تقرير القياس من الجهة</t>
         </r>
       </text>
     </comment>
@@ -103,24 +103,32 @@
     <comment ref="J7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/17 – تحديث
-استلام تقرير الملاحظات (7 ملاحظات)</t>
+          <t xml:space="preserve">2026/08/15 – تفتيش / زيارة ميدانية
+تفتيش دوري ورصد 5 ملاحظات على حفظ المصادر وسجلات الجرعات</t>
         </r>
       </text>
     </comment>
-    <comment ref="L7" authorId="0">
+    <comment ref="K7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/30 – إجراء
-معالجة 4 ملاحظات ورفع الشواهد</t>
+          <t xml:space="preserve">2026/08/22 – مراسلة
+إبلاغ المنشأة بالملاحظات ومهلة المعالجة</t>
         </r>
       </text>
     </comment>
-    <comment ref="N7" authorId="0">
+    <comment ref="M7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/16 – قرار
-اعتماد خطة معالجة الملاحظات المتبقية</t>
+          <t xml:space="preserve">2026/09/08 – تحديث
+استلام شواهد معالجة 4 ملاحظات</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O7" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">2026/09/21 – تفتيش / زيارة ميدانية
+زيارة تحقق ميدانية من المعالجة</t>
         </r>
       </text>
     </comment>
@@ -128,7 +136,7 @@
       <text>
         <r>
           <t xml:space="preserve">2026/09/29 – إقفال
-تمت معالجة جميع الملاحظات وإغلاقها من المراجعة الداخلية</t>
+التحقق من معالجة جميع الملاحظات وإغلاقها</t>
         </r>
       </text>
     </comment>
@@ -144,7 +152,7 @@
       <text>
         <r>
           <t xml:space="preserve">2026/09/02 – إجراء
-إعداد المواصفات الفنية</t>
+إعداد سيناريو التمرين وخطة التقييم</t>
         </r>
       </text>
     </comment>
@@ -152,7 +160,7 @@
       <text>
         <r>
           <t xml:space="preserve">2026/09/28 – متابعة
-تعليق الطلب بانتظار اعتماد الميزانية</t>
+تعليق موعد التمرين بانتظار تأكيد الجهات المشاركة</t>
         </r>
       </text>
     </comment>
@@ -168,7 +176,7 @@
       <text>
         <r>
           <t xml:space="preserve">2026/07/29 – إجراء
-توريد الأثاث والتجهيزات</t>
+حصر المصادر لدى الجهات المرخَّص لها ومطابقتها مع السجل</t>
         </r>
       </text>
     </comment>
@@ -176,7 +184,7 @@
       <text>
         <r>
           <t xml:space="preserve">2026/08/28 – إقفال
-تسليم القاعة وتشغيلها</t>
+اعتماد السجل المحدّث ونشره داخلياً</t>
         </r>
       </text>
     </comment>
@@ -185,7 +193,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="109">
   <si>
     <t>ملخص المواضيع</t>
   </si>
@@ -241,13 +249,13 @@
     <t>M-003</t>
   </si>
   <si>
-    <t>ربط النظام مع الجهة الخارجية</t>
-  </si>
-  <si>
-    <t>تقنية</t>
-  </si>
-  <si>
-    <t>تقنية المعلومات</t>
+    <t>تحديث لائحة الوقاية من الإشعاع</t>
+  </si>
+  <si>
+    <t>الأنظمة واللوائح</t>
+  </si>
+  <si>
+    <t>الإدارة القانونية</t>
   </si>
   <si>
     <t>خالد الشهري</t>
@@ -259,7 +267,7 @@
     <t>قيد الإجراء</t>
   </si>
   <si>
-    <t>استلام بيئة الاختبار</t>
+    <t>استلام 12 مرئية من الجهات</t>
   </si>
   <si>
     <t/>
@@ -268,13 +276,13 @@
     <t>M-001</t>
   </si>
   <si>
-    <t>تجديد عقد صيانة المبنى الرئيسي</t>
-  </si>
-  <si>
-    <t>عقود</t>
-  </si>
-  <si>
-    <t>إدارة المشتريات</t>
+    <t>استكمال متطلبات ترخيص منشأة طبية تستخدم مصادر مشعة</t>
+  </si>
+  <si>
+    <t>التراخيص والتصاريح</t>
+  </si>
+  <si>
+    <t>جهة طبية طالبة للترخيص</t>
   </si>
   <si>
     <t>أحمد العتيبي</t>
@@ -283,19 +291,19 @@
     <t>قيد الإجراء (متأخر)</t>
   </si>
   <si>
-    <t>متابعة التقييم الفني للعروض – بانتظار اجتماع لجنة الفحص</t>
+    <t>متابعة تنفيذ تعديلات الدروع – بانتظار تقرير القياس من الجهة</t>
   </si>
   <si>
     <t>M-005</t>
   </si>
   <si>
-    <t>تحديث سياسة العمل عن بعد</t>
-  </si>
-  <si>
-    <t>موارد بشرية</t>
-  </si>
-  <si>
-    <t>الموارد البشرية</t>
+    <t>إعداد التقرير السنوي للضمانات</t>
+  </si>
+  <si>
+    <t>الضمانات</t>
+  </si>
+  <si>
+    <t>إدارة الضمانات</t>
   </si>
   <si>
     <t>نورة الحربي</t>
@@ -313,13 +321,13 @@
     <t>M-002</t>
   </si>
   <si>
-    <t>معالجة ملاحظات المراجعة الداخلية</t>
-  </si>
-  <si>
-    <t>حوكمة</t>
-  </si>
-  <si>
-    <t>المراجعة الداخلية</t>
+    <t>معالجة ملاحظات التفتيش الدوري على منشأة صناعية</t>
+  </si>
+  <si>
+    <t>التفتيش والرقابة</t>
+  </si>
+  <si>
+    <t>منشأة صناعية مرخَّص لها</t>
   </si>
   <si>
     <t>سارة القحطاني</t>
@@ -331,19 +339,19 @@
     <t>مقفل</t>
   </si>
   <si>
-    <t>تمت معالجة جميع الملاحظات وإغلاقها من المراجعة الداخلية</t>
+    <t>التحقق من معالجة جميع الملاحظات وإغلاقها</t>
   </si>
   <si>
     <t>M-004</t>
   </si>
   <si>
-    <t>توريد أجهزة الحاسب للفرع الجديد</t>
-  </si>
-  <si>
-    <t>مشتريات</t>
-  </si>
-  <si>
-    <t>الشؤون المالية</t>
+    <t>تنفيذ تمرين الاستجابة لحادث إشعاعي</t>
+  </si>
+  <si>
+    <t>التأهب والاستجابة للطوارئ</t>
+  </si>
+  <si>
+    <t>الجهات المشاركة في الخطة الوطنية</t>
   </si>
   <si>
     <t>فهد الدوسري</t>
@@ -352,22 +360,22 @@
     <t>معلّق</t>
   </si>
   <si>
-    <t>تعليق الطلب بانتظار اعتماد الميزانية</t>
+    <t>تعليق موعد التمرين بانتظار تأكيد الجهات المشاركة</t>
   </si>
   <si>
     <t>M-006</t>
   </si>
   <si>
-    <t>تجهيز قاعة التدريب</t>
-  </si>
-  <si>
-    <t>مرافق</t>
-  </si>
-  <si>
-    <t>الخدمات العامة</t>
-  </si>
-  <si>
-    <t>تسليم القاعة وتشغيلها</t>
+    <t>تحديث السجل الوطني للمصادر المشعة</t>
+  </si>
+  <si>
+    <t>الوقاية من الإشعاع</t>
+  </si>
+  <si>
+    <t>إدارة الوقاية من الإشعاع</t>
+  </si>
+  <si>
+    <t>اعتماد السجل المحدّث ونشره داخلياً</t>
   </si>
   <si>
     <t>السجل الزمني للأحداث</t>
@@ -394,61 +402,67 @@
     <t>فتح الموضوع</t>
   </si>
   <si>
+    <t>اجتماع</t>
+  </si>
+  <si>
+    <t>ورشة عمل داخلية لمراجعة المسودة الأولى</t>
+  </si>
+  <si>
+    <t>إجراء</t>
+  </si>
+  <si>
+    <t>طرح المسودة لأخذ مرئيات الجهات ذات العلاقة</t>
+  </si>
+  <si>
+    <t>تحديث</t>
+  </si>
+  <si>
+    <t>تسجيل الموضوع: طلب ترخيص جديد لاستخدام مصادر مشعة في العلاج الإشعاعي، ويتطلب استيفاء متطلبات الدروع والتقييم الإشعاعي قبل إصدار الترخيص.</t>
+  </si>
+  <si>
     <t>مراسلة</t>
   </si>
   <si>
-    <t>مراسلة الجهة لطلب وثائق الربط</t>
-  </si>
-  <si>
-    <t>اجتماع</t>
-  </si>
-  <si>
-    <t>اجتماع فني مع فريق الجهة</t>
-  </si>
-  <si>
-    <t>تحديث</t>
-  </si>
-  <si>
-    <t>تسجيل الموضوع: انتهاء عقد الصيانة الحالي ويلزم الطرح والترسية قبل نهاية الربع لضمان استمرارية الخدمة.</t>
-  </si>
-  <si>
-    <t>إرسال خطاب لإدارة المشتريات بطلب طرح المنافسة</t>
-  </si>
-  <si>
-    <t>اجتماع مع المشتريات لمراجعة كراسة الشروط واعتماد نطاق العمل</t>
-  </si>
-  <si>
-    <t>لجنة العقود</t>
-  </si>
-  <si>
-    <t>إجراء</t>
-  </si>
-  <si>
-    <t>طرح المنافسة واستقبال ثلاثة عروض من المقاولين المؤهلين</t>
+    <t>إرسال خطاب للجهة بطلب استيفاء متطلبات الدروع وخطة الوقاية الإشعاعية</t>
+  </si>
+  <si>
+    <t>تفتيش / زيارة ميدانية</t>
+  </si>
+  <si>
+    <t>زيارة ميدانية للتحقق من غرفة العلاج وأنظمة الدروع؛ رُصدت 3 ملاحظات</t>
+  </si>
+  <si>
+    <t>فريق التفتيش</t>
+  </si>
+  <si>
+    <t>اجتماع مع الجهة لمناقشة خطة معالجة الملاحظات وجدولها الزمني</t>
+  </si>
+  <si>
+    <t>إدارة التراخيص</t>
   </si>
   <si>
     <t>متابعة</t>
   </si>
   <si>
-    <t>استلام تقرير الملاحظات (7 ملاحظات)</t>
-  </si>
-  <si>
-    <t>معالجة 4 ملاحظات ورفع الشواهد</t>
-  </si>
-  <si>
-    <t>قرار</t>
-  </si>
-  <si>
-    <t>اعتماد خطة معالجة الملاحظات المتبقية</t>
+    <t>تفتيش دوري ورصد 5 ملاحظات على حفظ المصادر وسجلات الجرعات</t>
+  </si>
+  <si>
+    <t>إبلاغ المنشأة بالملاحظات ومهلة المعالجة</t>
+  </si>
+  <si>
+    <t>استلام شواهد معالجة 4 ملاحظات</t>
+  </si>
+  <si>
+    <t>زيارة تحقق ميدانية من المعالجة</t>
   </si>
   <si>
     <t>إقفال</t>
   </si>
   <si>
-    <t>إعداد المواصفات الفنية</t>
-  </si>
-  <si>
-    <t>توريد الأثاث والتجهيزات</t>
+    <t>إعداد سيناريو التمرين وخطة التقييم</t>
+  </si>
+  <si>
+    <t>حصر المصادر لدى الجهات المرخَّص لها ومطابقتها مع السجل</t>
   </si>
   <si>
     <t>المخطط الزمني (Timeline) – عرض أسبوعي (يبدأ السبت)</t>
@@ -542,11 +556,11 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF64748B"/>
+      <color rgb="FF9333EA"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF9333EA"/>
+      <color rgb="FFD97706"/>
     </font>
     <font>
       <b/>
@@ -554,15 +568,15 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFD97706"/>
+      <color rgb="FF64748B"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F766E"/>
     </font>
     <font>
       <b/>
       <color rgb="FF0891B2"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFBE185D"/>
     </font>
     <font>
       <b/>
@@ -654,7 +668,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -715,31 +729,28 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -762,13 +773,13 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -776,6 +787,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -791,16 +805,16 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -811,10 +825,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1279,20 +1296,20 @@
         <v>23</v>
       </c>
       <c r="H4" s="8">
-        <v>46286</v>
+        <v>46256</v>
       </c>
       <c r="I4" s="8">
-        <v>46321</v>
+        <v>46312</v>
       </c>
       <c r="J4" s="8"/>
       <c r="K4" s="6">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="L4" s="6">
         <v>4</v>
       </c>
       <c r="M4" s="8">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="N4" s="6" t="s">
         <v>24</v>
@@ -1426,7 +1443,7 @@
         <v>48</v>
       </c>
       <c r="L7" s="6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M7" s="8">
         <v>46294</v>
@@ -1543,7 +1560,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -1613,7 +1630,7 @@
         <v>18</v>
       </c>
       <c r="C4" s="14">
-        <v>46286</v>
+        <v>46256</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>68</v>
@@ -1637,7 +1654,7 @@
         <v>18</v>
       </c>
       <c r="C5" s="14">
-        <v>46288</v>
+        <v>46261</v>
       </c>
       <c r="D5" s="16" t="s">
         <v>69</v>
@@ -1649,10 +1666,10 @@
         <v>25</v>
       </c>
       <c r="G5" s="13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H5" s="13">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1663,7 +1680,7 @@
         <v>18</v>
       </c>
       <c r="C6" s="14">
-        <v>46297</v>
+        <v>46276</v>
       </c>
       <c r="D6" s="17" t="s">
         <v>71</v>
@@ -1675,10 +1692,10 @@
         <v>25</v>
       </c>
       <c r="G6" s="13">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="H6" s="13">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1689,7 +1706,7 @@
         <v>18</v>
       </c>
       <c r="C7" s="14">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="D7" s="18" t="s">
         <v>73</v>
@@ -1701,10 +1718,10 @@
         <v>25</v>
       </c>
       <c r="G7" s="13">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="H7" s="13">
-        <v>7</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1742,10 +1759,10 @@
         <v>46271</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F9" s="19" t="s">
         <v>30</v>
@@ -1765,22 +1782,22 @@
         <v>27</v>
       </c>
       <c r="C10" s="20">
-        <v>46278</v>
+        <v>46280</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G10" s="19">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H10" s="19">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1794,19 +1811,19 @@
         <v>46291</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="G11" s="19">
         <v>25</v>
       </c>
       <c r="H11" s="19">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1820,7 +1837,7 @@
         <v>46300</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E12" s="19" t="s">
         <v>32</v>
@@ -1891,22 +1908,22 @@
         <v>42</v>
       </c>
       <c r="C15" s="20">
-        <v>46251</v>
-      </c>
-      <c r="D15" s="26" t="s">
-        <v>73</v>
+        <v>46249</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>77</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F15" s="19" t="s">
         <v>25</v>
       </c>
       <c r="G15" s="19">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H15" s="19">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1917,22 +1934,22 @@
         <v>42</v>
       </c>
       <c r="C16" s="20">
-        <v>46264</v>
-      </c>
-      <c r="D16" s="24" t="s">
-        <v>78</v>
+        <v>46256</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>75</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F16" s="19" t="s">
         <v>25</v>
       </c>
       <c r="G16" s="19">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="H16" s="19">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1943,19 +1960,19 @@
         <v>42</v>
       </c>
       <c r="C17" s="20">
-        <v>46281</v>
-      </c>
-      <c r="D17" s="27" t="s">
-        <v>83</v>
+        <v>46273</v>
+      </c>
+      <c r="D17" s="26" t="s">
+        <v>73</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F17" s="19" t="s">
         <v>25</v>
       </c>
       <c r="G17" s="19">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H17" s="19">
         <v>17</v>
@@ -1969,47 +1986,49 @@
         <v>42</v>
       </c>
       <c r="C18" s="20">
-        <v>46294</v>
-      </c>
-      <c r="D18" s="28" t="s">
-        <v>85</v>
+        <v>46286</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>77</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>48</v>
+        <v>86</v>
       </c>
       <c r="F18" s="19" t="s">
         <v>25</v>
       </c>
       <c r="G18" s="19">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="H18" s="19">
         <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" s="14">
-        <v>46254</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="F19" s="13" t="s">
+      <c r="A19" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="20">
+        <v>46294</v>
+      </c>
+      <c r="D19" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="F19" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="G19" s="13">
-        <v>0</v>
-      </c>
-      <c r="H19" s="13"/>
+      <c r="G19" s="19">
+        <v>48</v>
+      </c>
+      <c r="H19" s="19">
+        <v>8</v>
+      </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
@@ -2019,23 +2038,21 @@
         <v>50</v>
       </c>
       <c r="C20" s="14">
-        <v>46267</v>
-      </c>
-      <c r="D20" s="29" t="s">
-        <v>78</v>
+        <v>46254</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>68</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="F20" s="13" t="s">
         <v>25</v>
       </c>
       <c r="G20" s="13">
-        <v>13</v>
-      </c>
-      <c r="H20" s="13">
-        <v>13</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H20" s="13"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
@@ -2045,47 +2062,49 @@
         <v>50</v>
       </c>
       <c r="C21" s="14">
-        <v>46293</v>
-      </c>
-      <c r="D21" s="30" t="s">
-        <v>80</v>
+        <v>46267</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>71</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>55</v>
+        <v>88</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>25</v>
       </c>
       <c r="G21" s="13">
+        <v>13</v>
+      </c>
+      <c r="H21" s="13">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" s="14">
+        <v>46293</v>
+      </c>
+      <c r="D22" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="G22" s="13">
         <v>39</v>
       </c>
-      <c r="H21" s="13">
+      <c r="H22" s="13">
         <v>26</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="B22" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="C22" s="20">
-        <v>46218</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="E22" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="F22" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G22" s="19">
-        <v>0</v>
-      </c>
-      <c r="H22" s="19"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
@@ -2095,23 +2114,21 @@
         <v>57</v>
       </c>
       <c r="C23" s="20">
-        <v>46232</v>
-      </c>
-      <c r="D23" s="24" t="s">
-        <v>78</v>
+        <v>46218</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>68</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>87</v>
+        <v>40</v>
       </c>
       <c r="F23" s="19" t="s">
         <v>25</v>
       </c>
       <c r="G23" s="19">
-        <v>14</v>
-      </c>
-      <c r="H23" s="19">
-        <v>14</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H23" s="19"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
@@ -2121,21 +2138,47 @@
         <v>57</v>
       </c>
       <c r="C24" s="20">
-        <v>46262</v>
-      </c>
-      <c r="D24" s="28" t="s">
-        <v>85</v>
+        <v>46232</v>
+      </c>
+      <c r="D24" s="29" t="s">
+        <v>71</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="F24" s="19" t="s">
         <v>25</v>
       </c>
       <c r="G24" s="19">
+        <v>14</v>
+      </c>
+      <c r="H24" s="19">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C25" s="20">
+        <v>46262</v>
+      </c>
+      <c r="D25" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="E25" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="F25" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="G25" s="19">
         <v>44</v>
       </c>
-      <c r="H24" s="19">
+      <c r="H25" s="19">
         <v>30</v>
       </c>
     </row>
@@ -2161,48 +2204,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
-        <v>88</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="31"/>
-      <c r="N1" s="31"/>
-      <c r="O1" s="31"/>
-      <c r="P1" s="31"/>
-      <c r="Q1" s="31"/>
-      <c r="R1" s="31"/>
+      <c r="A1" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="30"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
-      <c r="R2" s="32"/>
+      <c r="A2" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
+      <c r="P2" s="31"/>
+      <c r="Q2" s="31"/>
+      <c r="R2" s="31"/>
     </row>
     <row r="3" ht="46" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
@@ -2217,256 +2260,258 @@
       <c r="D3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="33" t="s">
-        <v>90</v>
-      </c>
-      <c r="F3" s="33" t="s">
-        <v>91</v>
-      </c>
-      <c r="G3" s="33" t="s">
+      <c r="E3" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="H3" s="33" t="s">
+      <c r="F3" s="32" t="s">
         <v>93</v>
       </c>
-      <c r="I3" s="33" t="s">
+      <c r="G3" s="32" t="s">
         <v>94</v>
       </c>
-      <c r="J3" s="33" t="s">
+      <c r="H3" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="K3" s="33" t="s">
+      <c r="I3" s="32" t="s">
         <v>96</v>
       </c>
-      <c r="L3" s="33" t="s">
+      <c r="J3" s="32" t="s">
         <v>97</v>
       </c>
-      <c r="M3" s="33" t="s">
+      <c r="K3" s="32" t="s">
         <v>98</v>
       </c>
-      <c r="N3" s="33" t="s">
+      <c r="L3" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="O3" s="33" t="s">
+      <c r="M3" s="32" t="s">
         <v>100</v>
       </c>
-      <c r="P3" s="33" t="s">
+      <c r="N3" s="32" t="s">
         <v>101</v>
       </c>
-      <c r="Q3" s="33" t="s">
+      <c r="O3" s="32" t="s">
         <v>102</v>
       </c>
-      <c r="R3" s="34" t="s">
+      <c r="P3" s="32" t="s">
         <v>103</v>
       </c>
+      <c r="Q3" s="32" t="s">
+        <v>104</v>
+      </c>
+      <c r="R3" s="33" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="35">
-        <v>20</v>
-      </c>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="37"/>
-      <c r="I4" s="37"/>
-      <c r="J4" s="37"/>
-      <c r="K4" s="37"/>
-      <c r="L4" s="37"/>
-      <c r="M4" s="37"/>
-      <c r="N4" s="37"/>
-      <c r="O4" s="38" t="s">
-        <v>104</v>
-      </c>
-      <c r="P4" s="39" t="s">
-        <v>105</v>
-      </c>
+      <c r="D4" s="34">
+        <v>50</v>
+      </c>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="L4" s="38"/>
+      <c r="M4" s="39" t="s">
+        <v>107</v>
+      </c>
+      <c r="N4" s="38"/>
+      <c r="O4" s="38"/>
+      <c r="P4" s="38"/>
       <c r="Q4" s="40" t="s">
-        <v>105</v>
-      </c>
-      <c r="R4" s="41"/>
+        <v>107</v>
+      </c>
+      <c r="R4" s="38"/>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="36" t="s">
+      <c r="C5" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="35">
+      <c r="D5" s="34">
         <v>40</v>
       </c>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="37"/>
-      <c r="J5" s="37"/>
-      <c r="K5" s="37"/>
-      <c r="L5" s="42" t="s">
-        <v>105</v>
-      </c>
-      <c r="M5" s="38" t="s">
-        <v>105</v>
-      </c>
-      <c r="N5" s="39" t="s">
-        <v>105</v>
-      </c>
-      <c r="O5" s="41"/>
-      <c r="P5" s="43" t="s">
-        <v>105</v>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="M5" s="42" t="s">
+        <v>107</v>
+      </c>
+      <c r="N5" s="43" t="s">
+        <v>107</v>
+      </c>
+      <c r="O5" s="38"/>
+      <c r="P5" s="37" t="s">
+        <v>107</v>
       </c>
       <c r="Q5" s="44" t="s">
-        <v>105</v>
-      </c>
-      <c r="R5" s="41"/>
+        <v>107</v>
+      </c>
+      <c r="R5" s="38"/>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" s="35" t="s">
+      <c r="A6" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="34" t="s">
         <v>34</v>
       </c>
       <c r="C6" s="45" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="35">
+      <c r="D6" s="34">
         <v>8</v>
       </c>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="37"/>
-      <c r="J6" s="37"/>
-      <c r="K6" s="37"/>
-      <c r="L6" s="37"/>
-      <c r="M6" s="37"/>
-      <c r="N6" s="37"/>
-      <c r="O6" s="37"/>
-      <c r="P6" s="37"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="36"/>
+      <c r="H6" s="36"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="36"/>
+      <c r="K6" s="36"/>
+      <c r="L6" s="36"/>
+      <c r="M6" s="36"/>
+      <c r="N6" s="36"/>
+      <c r="O6" s="36"/>
+      <c r="P6" s="36"/>
       <c r="Q6" s="46" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="R6" s="47"/>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="34" t="s">
         <v>42</v>
       </c>
       <c r="C7" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="35">
+      <c r="D7" s="34">
         <v>48</v>
       </c>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
       <c r="I7" s="49" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="J7" s="50" t="s">
-        <v>105</v>
-      </c>
-      <c r="K7" s="51"/>
-      <c r="L7" s="52" t="s">
-        <v>105</v>
-      </c>
-      <c r="M7" s="51"/>
-      <c r="N7" s="53" t="s">
-        <v>105</v>
-      </c>
-      <c r="O7" s="51"/>
+        <v>107</v>
+      </c>
+      <c r="K7" s="51" t="s">
+        <v>107</v>
+      </c>
+      <c r="L7" s="52"/>
+      <c r="M7" s="53" t="s">
+        <v>107</v>
+      </c>
+      <c r="N7" s="52"/>
+      <c r="O7" s="50" t="s">
+        <v>107</v>
+      </c>
       <c r="P7" s="54" t="s">
-        <v>106</v>
-      </c>
-      <c r="Q7" s="37"/>
-      <c r="R7" s="37"/>
+        <v>108</v>
+      </c>
+      <c r="Q7" s="36"/>
+      <c r="R7" s="36"/>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A8" s="35" t="s">
+      <c r="A8" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="35" t="s">
+      <c r="B8" s="34" t="s">
         <v>50</v>
       </c>
       <c r="C8" s="55" t="s">
         <v>54</v>
       </c>
-      <c r="D8" s="35">
+      <c r="D8" s="34">
         <v>52</v>
       </c>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="37"/>
-      <c r="I8" s="37"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="36"/>
+      <c r="I8" s="36"/>
       <c r="J8" s="56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="K8" s="57"/>
       <c r="L8" s="58" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="M8" s="57"/>
       <c r="N8" s="57"/>
       <c r="O8" s="57"/>
       <c r="P8" s="59" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="Q8" s="57"/>
       <c r="R8" s="57"/>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="34" t="s">
         <v>57</v>
       </c>
       <c r="C9" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="D9" s="35">
+      <c r="D9" s="34">
         <v>44</v>
       </c>
       <c r="E9" s="49" t="s">
-        <v>105</v>
-      </c>
-      <c r="F9" s="51"/>
-      <c r="G9" s="52" t="s">
-        <v>105</v>
-      </c>
-      <c r="H9" s="51"/>
-      <c r="I9" s="51"/>
-      <c r="J9" s="51"/>
+        <v>107</v>
+      </c>
+      <c r="F9" s="52"/>
+      <c r="G9" s="60" t="s">
+        <v>107</v>
+      </c>
+      <c r="H9" s="52"/>
+      <c r="I9" s="52"/>
+      <c r="J9" s="52"/>
       <c r="K9" s="54" t="s">
-        <v>106</v>
-      </c>
-      <c r="L9" s="37"/>
-      <c r="M9" s="37"/>
-      <c r="N9" s="37"/>
-      <c r="O9" s="37"/>
-      <c r="P9" s="37"/>
-      <c r="Q9" s="37"/>
-      <c r="R9" s="37"/>
+        <v>108</v>
+      </c>
+      <c r="L9" s="36"/>
+      <c r="M9" s="36"/>
+      <c r="N9" s="36"/>
+      <c r="O9" s="36"/>
+      <c r="P9" s="36"/>
+      <c r="Q9" s="36"/>
+      <c r="R9" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Apply the official NRRC logo and brand colours
- Embed the official logo (horizontal and icon) extracted from the
  supplied vector file
- Formal letterhead uses the horizontal logo; icon in the app header and
  the other report styles; logo can be replaced or hidden
- Brand colours (green, gold, blue) as defaults across the app, the three
  report styles and the Excel export; refreshed samples

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vq5DRv9yx8RnT5NY8AHtK
</commit_message>
<xml_diff>
--- a/samples/5-ملف-Excel.xlsx
+++ b/samples/5-ملف-Excel.xlsx
@@ -539,7 +539,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF1F4E79"/>
+      <color rgb="FF066D39"/>
       <sz val="14"/>
     </font>
     <font>
@@ -597,7 +597,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E79"/>
+        <fgColor rgb="FF066D39"/>
       </patternFill>
     </fill>
     <fill>

</xml_diff>

<commit_message>
V2: event tool field and simplified event types
- Event type is now one of update / follow-up / action; a separate
  optional event tool records how it was done (letter, e-mail, phone
  call, meeting, decision, field visit, other), also on closing
- Tool shown with an icon in the app timeline and all report styles,
  as its own column in the action log and in the Excel event sheet
- Existing data is migrated on load and on restore (e.g. meeting ->
  action + meeting tool); unknown types fall back safely
- Version bumped to V2; refreshed samples

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vq5DRv9yx8RnT5NY8AHtK
</commit_message>
<xml_diff>
--- a/samples/5-ملف-Excel.xlsx
+++ b/samples/5-ملف-Excel.xlsx
@@ -23,7 +23,7 @@
         <r>
           <t xml:space="preserve">2026/08/22 – فتح الموضوع
 تسجيل الموضوع
-2026/08/27 – اجتماع
+2026/08/27 – إجراء · اجتماع
 ورشة عمل داخلية لمراجعة المسودة الأولى</t>
         </r>
       </text>
@@ -39,7 +39,7 @@
     <comment ref="Q4" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/10/07 – تحديث
+          <t xml:space="preserve">2026/10/07 – تحديث · بريد إلكتروني
 استلام 12 مرئية من الجهات</t>
         </r>
       </text>
@@ -55,7 +55,7 @@
     <comment ref="M5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/06 – مراسلة (أحمد العتيبي)
+          <t xml:space="preserve">2026/09/06 – متابعة · خطاب (أحمد العتيبي)
 إرسال خطاب للجهة بطلب استيفاء متطلبات الدروع وخطة الوقاية الإشعاعية</t>
         </r>
       </text>
@@ -63,7 +63,7 @@
     <comment ref="N5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/15 – تفتيش / زيارة ميدانية (فريق التفتيش)
+          <t xml:space="preserve">2026/09/15 – إجراء · زيارة ميدانية (فريق التفتيش)
 زيارة ميدانية للتحقق من غرفة العلاج وأنظمة الدروع؛ رُصدت 3 ملاحظات</t>
         </r>
       </text>
@@ -71,7 +71,7 @@
     <comment ref="P5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/26 – اجتماع (إدارة التراخيص)
+          <t xml:space="preserve">2026/09/26 – إجراء · اجتماع (إدارة التراخيص)
 اجتماع مع الجهة لمناقشة خطة معالجة الملاحظات وجدولها الزمني</t>
         </r>
       </text>
@@ -79,7 +79,7 @@
     <comment ref="Q5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/10/05 – متابعة (أحمد العتيبي)
+          <t xml:space="preserve">2026/10/05 – متابعة · اتصال هاتفي (أحمد العتيبي)
 متابعة تنفيذ تعديلات الدروع – بانتظار تقرير القياس من الجهة</t>
         </r>
       </text>
@@ -103,7 +103,7 @@
     <comment ref="J7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/15 – تفتيش / زيارة ميدانية
+          <t xml:space="preserve">2026/08/15 – إجراء · زيارة ميدانية
 تفتيش دوري ورصد 5 ملاحظات على حفظ المصادر وسجلات الجرعات</t>
         </r>
       </text>
@@ -111,7 +111,7 @@
     <comment ref="K7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/22 – مراسلة
+          <t xml:space="preserve">2026/08/22 – متابعة · خطاب
 إبلاغ المنشأة بالملاحظات ومهلة المعالجة</t>
         </r>
       </text>
@@ -119,7 +119,7 @@
     <comment ref="M7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/08 – تحديث
+          <t xml:space="preserve">2026/09/08 – تحديث · بريد إلكتروني
 استلام شواهد معالجة 4 ملاحظات</t>
         </r>
       </text>
@@ -127,7 +127,7 @@
     <comment ref="O7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/21 – تفتيش / زيارة ميدانية
+          <t xml:space="preserve">2026/09/21 – إجراء · زيارة ميدانية
 زيارة تحقق ميدانية من المعالجة</t>
         </r>
       </text>
@@ -193,7 +193,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="112">
   <si>
     <t>ملخص المواضيع</t>
   </si>
@@ -387,6 +387,9 @@
     <t>نوع الحدث</t>
   </si>
   <si>
+    <t>أداة الحدث</t>
+  </si>
+  <si>
     <t>ما تم</t>
   </si>
   <si>
@@ -402,31 +405,37 @@
     <t>فتح الموضوع</t>
   </si>
   <si>
+    <t>إجراء</t>
+  </si>
+  <si>
     <t>اجتماع</t>
   </si>
   <si>
     <t>ورشة عمل داخلية لمراجعة المسودة الأولى</t>
   </si>
   <si>
-    <t>إجراء</t>
-  </si>
-  <si>
     <t>طرح المسودة لأخذ مرئيات الجهات ذات العلاقة</t>
   </si>
   <si>
     <t>تحديث</t>
   </si>
   <si>
+    <t>بريد إلكتروني</t>
+  </si>
+  <si>
     <t>تسجيل الموضوع: طلب ترخيص جديد لاستخدام مصادر مشعة في العلاج الإشعاعي، ويتطلب استيفاء متطلبات الدروع والتقييم الإشعاعي قبل إصدار الترخيص.</t>
   </si>
   <si>
-    <t>مراسلة</t>
+    <t>متابعة</t>
+  </si>
+  <si>
+    <t>خطاب</t>
   </si>
   <si>
     <t>إرسال خطاب للجهة بطلب استيفاء متطلبات الدروع وخطة الوقاية الإشعاعية</t>
   </si>
   <si>
-    <t>تفتيش / زيارة ميدانية</t>
+    <t>زيارة ميدانية</t>
   </si>
   <si>
     <t>زيارة ميدانية للتحقق من غرفة العلاج وأنظمة الدروع؛ رُصدت 3 ملاحظات</t>
@@ -441,7 +450,7 @@
     <t>إدارة التراخيص</t>
   </si>
   <si>
-    <t>متابعة</t>
+    <t>اتصال هاتفي</t>
   </si>
   <si>
     <t>تفتيش دوري ورصد 5 ملاحظات على حفظ المصادر وسجلات الجرعات</t>
@@ -529,7 +538,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -556,23 +565,11 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF9333EA"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FFD97706"/>
     </font>
     <font>
       <b/>
       <color rgb="FF2563EB"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF64748B"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF0F766E"/>
     </font>
     <font>
       <b/>
@@ -668,7 +665,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -717,50 +714,38 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -777,19 +762,10 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -805,19 +781,19 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -825,13 +801,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1560,19 +1533,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="13" style="1" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="70" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="66" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>61</v>
       </c>
@@ -1583,8 +1557,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="2"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1595,8 +1570,9 @@
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1621,8 +1597,11 @@
       <c r="H3" s="4" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>17</v>
       </c>
@@ -1633,20 +1612,23 @@
         <v>46256</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E4" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" s="13">
+      <c r="G4" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="13">
         <v>0</v>
       </c>
-      <c r="H4" s="13"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I4" s="13"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>17</v>
       </c>
@@ -1657,22 +1639,25 @@
         <v>46261</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5" s="13">
-        <v>5</v>
+        <v>72</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>25</v>
       </c>
       <c r="H5" s="13">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I5" s="13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>17</v>
       </c>
@@ -1682,23 +1667,26 @@
       <c r="C6" s="14">
         <v>46276</v>
       </c>
-      <c r="D6" s="17" t="s">
-        <v>71</v>
+      <c r="D6" s="16" t="s">
+        <v>70</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="G6" s="13">
+        <v>73</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="13">
         <v>20</v>
       </c>
-      <c r="H6" s="13">
+      <c r="I6" s="13">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>17</v>
       </c>
@@ -1708,151 +1696,169 @@
       <c r="C7" s="14">
         <v>46302</v>
       </c>
-      <c r="D7" s="18" t="s">
-        <v>73</v>
+      <c r="D7" s="17" t="s">
+        <v>74</v>
       </c>
       <c r="E7" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="F7" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" s="13">
+      <c r="G7" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="13">
         <v>46</v>
       </c>
-      <c r="H7" s="13">
+      <c r="I7" s="13">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="20">
+      <c r="C8" s="19">
         <v>46266</v>
       </c>
-      <c r="D8" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="E8" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="F8" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="19">
+      <c r="D8" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="18">
         <v>0</v>
       </c>
-      <c r="H8" s="19"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="I8" s="18"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="20">
+      <c r="C9" s="19">
         <v>46271</v>
       </c>
-      <c r="D9" s="22" t="s">
-        <v>75</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="F9" s="19" t="s">
+      <c r="D9" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="G9" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="19">
+      <c r="H9" s="18">
         <v>5</v>
       </c>
-      <c r="H9" s="19">
+      <c r="I9" s="18">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="20">
+      <c r="C10" s="19">
         <v>46280</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="D10" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="G10" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="H10" s="18">
+        <v>14</v>
+      </c>
+      <c r="I10" s="18">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="19">
+        <v>46291</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="H11" s="18">
+        <v>25</v>
+      </c>
+      <c r="I11" s="18">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="19">
+        <v>46300</v>
+      </c>
+      <c r="D12" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="E10" s="19" t="s">
-        <v>78</v>
-      </c>
-      <c r="F10" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="G10" s="19">
-        <v>14</v>
-      </c>
-      <c r="H10" s="19">
+      <c r="E12" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="F12" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="G12" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="H12" s="18">
+        <v>34</v>
+      </c>
+      <c r="I12" s="18">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="20">
-        <v>46291</v>
-      </c>
-      <c r="D11" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="F11" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="G11" s="19">
-        <v>25</v>
-      </c>
-      <c r="H11" s="19">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="20">
-        <v>46300</v>
-      </c>
-      <c r="D12" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="F12" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="G12" s="19">
-        <v>34</v>
-      </c>
-      <c r="H12" s="19">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>33</v>
       </c>
@@ -1863,174 +1869,195 @@
         <v>46298</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E13" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="F13" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="G13" s="13">
+      <c r="G13" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="13">
         <v>0</v>
       </c>
-      <c r="H13" s="13"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
+      <c r="I13" s="13"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="20">
+      <c r="C14" s="19">
         <v>46246</v>
       </c>
-      <c r="D14" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="E14" s="19" t="s">
+      <c r="D14" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="F14" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G14" s="19">
+      <c r="G14" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H14" s="18">
         <v>0</v>
       </c>
-      <c r="H14" s="19"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+      <c r="I14" s="18"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="19">
         <v>46249</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" s="18">
+        <v>3</v>
+      </c>
+      <c r="I15" s="18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="19">
+        <v>46256</v>
+      </c>
+      <c r="D16" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="E15" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="F15" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" s="19">
-        <v>3</v>
-      </c>
-      <c r="H15" s="19">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="19" t="s">
+      <c r="E16" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H16" s="18">
+        <v>10</v>
+      </c>
+      <c r="I16" s="18">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B17" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="20">
-        <v>46256</v>
-      </c>
-      <c r="D16" s="22" t="s">
+      <c r="C17" s="19">
+        <v>46273</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="E17" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E16" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="F16" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G16" s="19">
-        <v>10</v>
-      </c>
-      <c r="H16" s="19">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
+      <c r="F17" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="G17" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H17" s="18">
+        <v>27</v>
+      </c>
+      <c r="I17" s="18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B18" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="20">
-        <v>46273</v>
-      </c>
-      <c r="D17" s="26" t="s">
-        <v>73</v>
-      </c>
-      <c r="E17" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="F17" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G17" s="19">
-        <v>27</v>
-      </c>
-      <c r="H17" s="19">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="19" t="s">
+      <c r="C18" s="19">
+        <v>46286</v>
+      </c>
+      <c r="D18" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="G18" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H18" s="18">
+        <v>40</v>
+      </c>
+      <c r="I18" s="18">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B19" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="20">
-        <v>46286</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>77</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="F18" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G18" s="19">
-        <v>40</v>
-      </c>
-      <c r="H18" s="19">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="C19" s="20">
+      <c r="C19" s="19">
         <v>46294</v>
       </c>
-      <c r="D19" s="27" t="s">
-        <v>87</v>
-      </c>
-      <c r="E19" s="19" t="s">
+      <c r="D19" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="F19" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="F19" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G19" s="19">
+      <c r="G19" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H19" s="18">
         <v>48</v>
       </c>
-      <c r="H19" s="19">
+      <c r="I19" s="18">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>49</v>
       </c>
@@ -2041,20 +2068,23 @@
         <v>46254</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E20" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="F20" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="G20" s="13">
+      <c r="G20" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H20" s="13">
         <v>0</v>
       </c>
-      <c r="H20" s="13"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I20" s="13"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
         <v>49</v>
       </c>
@@ -2064,23 +2094,26 @@
       <c r="C21" s="14">
         <v>46267</v>
       </c>
-      <c r="D21" s="17" t="s">
-        <v>71</v>
+      <c r="D21" s="16" t="s">
+        <v>70</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>88</v>
+        <v>25</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="G21" s="13">
-        <v>13</v>
+        <v>91</v>
+      </c>
+      <c r="G21" s="13" t="s">
+        <v>25</v>
       </c>
       <c r="H21" s="13">
         <v>13</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I21" s="13">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
         <v>49</v>
       </c>
@@ -2090,103 +2123,115 @@
       <c r="C22" s="14">
         <v>46293</v>
       </c>
-      <c r="D22" s="28" t="s">
-        <v>82</v>
+      <c r="D22" s="25" t="s">
+        <v>77</v>
       </c>
       <c r="E22" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="F22" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="F22" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="G22" s="13">
+      <c r="G22" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H22" s="13">
         <v>39</v>
       </c>
-      <c r="H22" s="13">
+      <c r="I22" s="13">
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="19" t="s">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="C23" s="20">
+      <c r="C23" s="19">
         <v>46218</v>
       </c>
-      <c r="D23" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="E23" s="19" t="s">
+      <c r="D23" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="F23" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G23" s="19">
+      <c r="G23" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H23" s="18">
         <v>0</v>
       </c>
-      <c r="H23" s="19"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
+      <c r="I23" s="18"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="20">
+      <c r="C24" s="19">
         <v>46232</v>
       </c>
-      <c r="D24" s="29" t="s">
-        <v>71</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="F24" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G24" s="19">
+      <c r="D24" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="E24" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="G24" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H24" s="18">
         <v>14</v>
       </c>
-      <c r="H24" s="19">
+      <c r="I24" s="18">
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="19" t="s">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="19">
         <v>46262</v>
       </c>
-      <c r="D25" s="27" t="s">
-        <v>87</v>
-      </c>
-      <c r="E25" s="19" t="s">
+      <c r="D25" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="F25" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="F25" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="G25" s="19">
+      <c r="G25" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H25" s="18">
         <v>44</v>
       </c>
-      <c r="H25" s="19">
+      <c r="I25" s="18">
         <v>30</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H3"/>
+  <autoFilter ref="A3:I3"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2204,48 +2249,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
+      <c r="A1" s="26" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
+      <c r="Q1" s="26"/>
+      <c r="R1" s="26"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="31" t="s">
-        <v>91</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="31"/>
-      <c r="Q2" s="31"/>
-      <c r="R2" s="31"/>
+      <c r="A2" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
     </row>
     <row r="3" ht="46" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
@@ -2260,258 +2305,258 @@
       <c r="D3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="F3" s="32" t="s">
-        <v>93</v>
-      </c>
-      <c r="G3" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="H3" s="32" t="s">
+      <c r="E3" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="I3" s="32" t="s">
+      <c r="F3" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="J3" s="32" t="s">
+      <c r="G3" s="28" t="s">
         <v>97</v>
       </c>
-      <c r="K3" s="32" t="s">
+      <c r="H3" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="L3" s="32" t="s">
+      <c r="I3" s="28" t="s">
         <v>99</v>
       </c>
-      <c r="M3" s="32" t="s">
+      <c r="J3" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="N3" s="32" t="s">
+      <c r="K3" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="O3" s="32" t="s">
+      <c r="L3" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="P3" s="32" t="s">
+      <c r="M3" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="Q3" s="32" t="s">
+      <c r="N3" s="28" t="s">
         <v>104</v>
       </c>
-      <c r="R3" s="33" t="s">
+      <c r="O3" s="28" t="s">
         <v>105</v>
       </c>
+      <c r="P3" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q3" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="R3" s="29" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="C4" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="34">
+      <c r="D4" s="30">
         <v>50</v>
       </c>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="37" t="s">
-        <v>106</v>
-      </c>
-      <c r="L4" s="38"/>
-      <c r="M4" s="39" t="s">
-        <v>107</v>
-      </c>
-      <c r="N4" s="38"/>
-      <c r="O4" s="38"/>
-      <c r="P4" s="38"/>
-      <c r="Q4" s="40" t="s">
-        <v>107</v>
-      </c>
-      <c r="R4" s="38"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="33" t="s">
+        <v>109</v>
+      </c>
+      <c r="L4" s="34"/>
+      <c r="M4" s="33" t="s">
+        <v>110</v>
+      </c>
+      <c r="N4" s="34"/>
+      <c r="O4" s="34"/>
+      <c r="P4" s="34"/>
+      <c r="Q4" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="R4" s="34"/>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="34">
+      <c r="D5" s="30">
         <v>40</v>
       </c>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36"/>
-      <c r="L5" s="41" t="s">
-        <v>107</v>
-      </c>
-      <c r="M5" s="42" t="s">
-        <v>107</v>
-      </c>
-      <c r="N5" s="43" t="s">
-        <v>107</v>
-      </c>
-      <c r="O5" s="38"/>
-      <c r="P5" s="37" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q5" s="44" t="s">
-        <v>107</v>
-      </c>
-      <c r="R5" s="38"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="36" t="s">
+        <v>110</v>
+      </c>
+      <c r="M5" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="N5" s="33" t="s">
+        <v>110</v>
+      </c>
+      <c r="O5" s="34"/>
+      <c r="P5" s="33" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q5" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="R5" s="34"/>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="45" t="s">
+      <c r="C6" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="34">
+      <c r="D6" s="30">
         <v>8</v>
       </c>
-      <c r="E6" s="36"/>
-      <c r="F6" s="36"/>
-      <c r="G6" s="36"/>
-      <c r="H6" s="36"/>
-      <c r="I6" s="36"/>
-      <c r="J6" s="36"/>
-      <c r="K6" s="36"/>
-      <c r="L6" s="36"/>
-      <c r="M6" s="36"/>
-      <c r="N6" s="36"/>
-      <c r="O6" s="36"/>
-      <c r="P6" s="36"/>
-      <c r="Q6" s="46" t="s">
-        <v>107</v>
-      </c>
-      <c r="R6" s="47"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="32"/>
+      <c r="N6" s="32"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="32"/>
+      <c r="Q6" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="R6" s="40"/>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="34">
+      <c r="D7" s="30">
         <v>48</v>
       </c>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="J7" s="50" t="s">
-        <v>107</v>
-      </c>
-      <c r="K7" s="51" t="s">
-        <v>107</v>
-      </c>
-      <c r="L7" s="52"/>
-      <c r="M7" s="53" t="s">
-        <v>107</v>
-      </c>
-      <c r="N7" s="52"/>
-      <c r="O7" s="50" t="s">
-        <v>107</v>
-      </c>
-      <c r="P7" s="54" t="s">
-        <v>108</v>
-      </c>
-      <c r="Q7" s="36"/>
-      <c r="R7" s="36"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="42" t="s">
+        <v>110</v>
+      </c>
+      <c r="J7" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="K7" s="44" t="s">
+        <v>110</v>
+      </c>
+      <c r="L7" s="45"/>
+      <c r="M7" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="N7" s="45"/>
+      <c r="O7" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="P7" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q7" s="32"/>
+      <c r="R7" s="32"/>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="55" t="s">
+      <c r="C8" s="48" t="s">
         <v>54</v>
       </c>
-      <c r="D8" s="34">
+      <c r="D8" s="30">
         <v>52</v>
       </c>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="36"/>
-      <c r="J8" s="56" t="s">
-        <v>107</v>
-      </c>
-      <c r="K8" s="57"/>
-      <c r="L8" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="M8" s="57"/>
-      <c r="N8" s="57"/>
-      <c r="O8" s="57"/>
-      <c r="P8" s="59" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q8" s="57"/>
-      <c r="R8" s="57"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="49" t="s">
+        <v>110</v>
+      </c>
+      <c r="K8" s="50"/>
+      <c r="L8" s="51" t="s">
+        <v>110</v>
+      </c>
+      <c r="M8" s="50"/>
+      <c r="N8" s="50"/>
+      <c r="O8" s="50"/>
+      <c r="P8" s="52" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q8" s="50"/>
+      <c r="R8" s="50"/>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="D9" s="34">
+      <c r="D9" s="30">
         <v>44</v>
       </c>
-      <c r="E9" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="F9" s="52"/>
-      <c r="G9" s="60" t="s">
-        <v>107</v>
-      </c>
-      <c r="H9" s="52"/>
-      <c r="I9" s="52"/>
-      <c r="J9" s="52"/>
-      <c r="K9" s="54" t="s">
-        <v>108</v>
-      </c>
-      <c r="L9" s="36"/>
-      <c r="M9" s="36"/>
-      <c r="N9" s="36"/>
-      <c r="O9" s="36"/>
-      <c r="P9" s="36"/>
-      <c r="Q9" s="36"/>
-      <c r="R9" s="36"/>
+      <c r="E9" s="42" t="s">
+        <v>110</v>
+      </c>
+      <c r="F9" s="45"/>
+      <c r="G9" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="H9" s="45"/>
+      <c r="I9" s="45"/>
+      <c r="J9" s="45"/>
+      <c r="K9" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="L9" s="32"/>
+      <c r="M9" s="32"/>
+      <c r="N9" s="32"/>
+      <c r="O9" s="32"/>
+      <c r="P9" s="32"/>
+      <c r="Q9" s="32"/>
+      <c r="R9" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
V4: executor and recipient fields; formal report wording
- Event and closing forms: separate executor and recipient fields with
  suggestions from names already used
- Formal report: topic page heading is the topic title only, first
  section renamed to 'البيانات', action log gets a recipient column
  after the executor column; tighter topic page spacing
- Consulting and modern styles show executor and recipient; Excel event
  sheet has separate executor and recipient columns
- Version V4; refreshed samples

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vq5DRv9yx8RnT5NY8AHtK
</commit_message>
<xml_diff>
--- a/samples/5-ملف-Excel.xlsx
+++ b/samples/5-ملف-Excel.xlsx
@@ -21,17 +21,17 @@
     <comment ref="K4" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/22 – فتح الموضوع
+          <t xml:space="preserve">2026/08/23 – فتح الموضوع
 تسجيل الموضوع
-2026/08/27 – إجراء · اجتماع
+2026/08/28 – إجراء · اجتماع
 ورشة عمل داخلية لمراجعة المسودة الأولى</t>
         </r>
       </text>
     </comment>
-    <comment ref="M4" authorId="0">
+    <comment ref="N4" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/11 – إجراء
+          <t xml:space="preserve">2026/09/12 – إجراء
 طرح المسودة لأخذ مرئيات الجهات ذات العلاقة</t>
         </r>
       </text>
@@ -39,7 +39,7 @@
     <comment ref="Q4" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/10/07 – تحديث · بريد إلكتروني
+          <t xml:space="preserve">2026/10/08 – تحديث · بريد إلكتروني
 استلام 12 مرئية من الجهات</t>
         </r>
       </text>
@@ -47,7 +47,7 @@
     <comment ref="L5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/01 – فتح الموضوع
+          <t xml:space="preserve">2026/09/02 – فتح الموضوع
 تسجيل الموضوع: طلب ترخيص جديد لاستخدام مصادر مشعة في العلاج الإشعاعي، ويتطلب استيفاء متطلبات الدروع والتقييم الإشعاعي قبل إصدار الترخيص.</t>
         </r>
       </text>
@@ -55,7 +55,7 @@
     <comment ref="M5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/06 – متابعة · خطاب (أحمد العتيبي)
+          <t xml:space="preserve">2026/09/07 – متابعة · خطاب – المنفذ: أحمد العتيبي – المستلم: جهة طبية طالبة للترخيص
 إرسال خطاب للجهة بطلب استيفاء متطلبات الدروع وخطة الوقاية الإشعاعية</t>
         </r>
       </text>
@@ -63,7 +63,7 @@
     <comment ref="N5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/15 – إجراء · زيارة ميدانية (فريق التفتيش)
+          <t xml:space="preserve">2026/09/16 – إجراء · زيارة ميدانية – المنفذ: فريق التفتيش
 زيارة ميدانية للتحقق من غرفة العلاج وأنظمة الدروع؛ رُصدت 3 ملاحظات</t>
         </r>
       </text>
@@ -71,7 +71,7 @@
     <comment ref="P5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/26 – إجراء · اجتماع (إدارة التراخيص)
+          <t xml:space="preserve">2026/09/27 – إجراء · اجتماع – المنفذ: إدارة التراخيص – المستلم: جهة طبية طالبة للترخيص
 اجتماع مع الجهة لمناقشة خطة معالجة الملاحظات وجدولها الزمني</t>
         </r>
       </text>
@@ -79,7 +79,7 @@
     <comment ref="Q5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/10/05 – متابعة · اتصال هاتفي (أحمد العتيبي)
+          <t xml:space="preserve">2026/10/06 – متابعة · اتصال هاتفي – المنفذ: أحمد العتيبي – المستلم: مسؤول الوقاية الإشعاعية بالجهة
 متابعة تنفيذ تعديلات الدروع – بانتظار تقرير القياس من الجهة</t>
         </r>
       </text>
@@ -87,7 +87,7 @@
     <comment ref="Q6" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/10/03 – فتح الموضوع
+          <t xml:space="preserve">2026/10/04 – فتح الموضوع
 تسجيل الموضوع</t>
         </r>
       </text>
@@ -95,7 +95,7 @@
     <comment ref="I7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/12 – فتح الموضوع
+          <t xml:space="preserve">2026/08/13 – فتح الموضوع
 تسجيل الموضوع</t>
         </r>
       </text>
@@ -103,7 +103,7 @@
     <comment ref="J7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/15 – إجراء · زيارة ميدانية
+          <t xml:space="preserve">2026/08/16 – إجراء · زيارة ميدانية
 تفتيش دوري ورصد 5 ملاحظات على حفظ المصادر وسجلات الجرعات</t>
         </r>
       </text>
@@ -111,7 +111,7 @@
     <comment ref="K7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/22 – متابعة · خطاب
+          <t xml:space="preserve">2026/08/23 – متابعة · خطاب – المنفذ: سارة القحطاني – المستلم: منشأة صناعية مرخَّص لها
 إبلاغ المنشأة بالملاحظات ومهلة المعالجة</t>
         </r>
       </text>
@@ -119,7 +119,7 @@
     <comment ref="M7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/08 – تحديث · بريد إلكتروني
+          <t xml:space="preserve">2026/09/09 – تحديث · بريد إلكتروني
 استلام شواهد معالجة 4 ملاحظات</t>
         </r>
       </text>
@@ -127,7 +127,7 @@
     <comment ref="O7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/21 – إجراء · زيارة ميدانية
+          <t xml:space="preserve">2026/09/22 – إجراء · زيارة ميدانية
 زيارة تحقق ميدانية من المعالجة</t>
         </r>
       </text>
@@ -135,7 +135,7 @@
     <comment ref="P7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/29 – إقفال
+          <t xml:space="preserve">2026/09/30 – إقفال
 التحقق من معالجة جميع الملاحظات وإغلاقها</t>
         </r>
       </text>
@@ -143,7 +143,7 @@
     <comment ref="J8" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/20 – فتح الموضوع
+          <t xml:space="preserve">2026/08/21 – فتح الموضوع
 تسجيل الموضوع</t>
         </r>
       </text>
@@ -151,7 +151,7 @@
     <comment ref="L8" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/02 – إجراء
+          <t xml:space="preserve">2026/09/03 – إجراء
 إعداد سيناريو التمرين وخطة التقييم</t>
         </r>
       </text>
@@ -159,7 +159,7 @@
     <comment ref="P8" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/28 – متابعة
+          <t xml:space="preserve">2026/09/29 – متابعة
 تعليق موعد التمرين بانتظار تأكيد الجهات المشاركة</t>
         </r>
       </text>
@@ -167,7 +167,7 @@
     <comment ref="E9" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/07/15 – فتح الموضوع
+          <t xml:space="preserve">2026/07/16 – فتح الموضوع
 تسجيل الموضوع</t>
         </r>
       </text>
@@ -175,15 +175,15 @@
     <comment ref="G9" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/07/29 – إجراء
+          <t xml:space="preserve">2026/07/30 – إجراء
 حصر المصادر لدى الجهات المرخَّص لها ومطابقتها مع السجل</t>
         </r>
       </text>
     </comment>
-    <comment ref="K9" authorId="0">
+    <comment ref="L9" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/28 – إقفال
+          <t xml:space="preserve">2026/08/29 – إقفال
 اعتماد السجل المحدّث ونشره داخلياً</t>
         </r>
       </text>
@@ -193,12 +193,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="114">
   <si>
     <t>ملخص المواضيع</t>
   </si>
   <si>
-    <t>تاريخ الإصدار: 2026/10/11</t>
+    <t>تاريخ الإصدار: 2026/10/12</t>
   </si>
   <si>
     <t>المرجع</t>
@@ -393,7 +393,10 @@
     <t>ما تم</t>
   </si>
   <si>
-    <t>بواسطة</t>
+    <t>المنفذ</t>
+  </si>
+  <si>
+    <t>المستلم</t>
   </si>
   <si>
     <t>اليوم من الفتح</t>
@@ -451,6 +454,9 @@
   </si>
   <si>
     <t>اتصال هاتفي</t>
+  </si>
+  <si>
+    <t>مسؤول الوقاية الإشعاعية بالجهة</t>
   </si>
   <si>
     <t>تفتيش دوري ورصد 5 ملاحظات على حفظ المصادر وسجلات الجرعات</t>
@@ -1269,10 +1275,10 @@
         <v>23</v>
       </c>
       <c r="H4" s="8">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="I4" s="8">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="J4" s="8"/>
       <c r="K4" s="6">
@@ -1282,7 +1288,7 @@
         <v>4</v>
       </c>
       <c r="M4" s="8">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="N4" s="6" t="s">
         <v>24</v>
@@ -1314,10 +1320,10 @@
         <v>31</v>
       </c>
       <c r="H5" s="8">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="I5" s="8">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="J5" s="8"/>
       <c r="K5" s="6">
@@ -1327,7 +1333,7 @@
         <v>5</v>
       </c>
       <c r="M5" s="8">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="N5" s="6" t="s">
         <v>32</v>
@@ -1359,10 +1365,10 @@
         <v>39</v>
       </c>
       <c r="H6" s="8">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="I6" s="8">
-        <v>46341</v>
+        <v>46342</v>
       </c>
       <c r="J6" s="8"/>
       <c r="K6" s="6">
@@ -1372,7 +1378,7 @@
         <v>1</v>
       </c>
       <c r="M6" s="8">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="N6" s="6" t="s">
         <v>40</v>
@@ -1404,13 +1410,13 @@
         <v>47</v>
       </c>
       <c r="H7" s="8">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="I7" s="8">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="J7" s="8">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="K7" s="6">
         <v>48</v>
@@ -1419,7 +1425,7 @@
         <v>6</v>
       </c>
       <c r="M7" s="8">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="N7" s="6" t="s">
         <v>48</v>
@@ -1451,10 +1457,10 @@
         <v>54</v>
       </c>
       <c r="H8" s="8">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="I8" s="8">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="J8" s="8"/>
       <c r="K8" s="6">
@@ -1464,7 +1470,7 @@
         <v>3</v>
       </c>
       <c r="M8" s="8">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="N8" s="6" t="s">
         <v>55</v>
@@ -1496,13 +1502,13 @@
         <v>47</v>
       </c>
       <c r="H9" s="8">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="I9" s="8">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="J9" s="8">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="K9" s="6">
         <v>44</v>
@@ -1511,7 +1517,7 @@
         <v>3</v>
       </c>
       <c r="M9" s="8">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="N9" s="6" t="s">
         <v>60</v>
@@ -1533,20 +1539,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="13" style="1" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="66" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="6" max="6" width="58" customWidth="1"/>
+    <col min="7" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>61</v>
       </c>
@@ -1558,8 +1564,9 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1571,8 +1578,9 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J2" s="3"/>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1600,8 +1608,11 @@
       <c r="I3" s="4" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J3" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>17</v>
       </c>
@@ -1609,10 +1620,10 @@
         <v>18</v>
       </c>
       <c r="C4" s="14">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>25</v>
@@ -1623,12 +1634,15 @@
       <c r="G4" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="13">
+      <c r="H4" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="13">
         <v>0</v>
       </c>
-      <c r="I4" s="13"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J4" s="13"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>17</v>
       </c>
@@ -1636,28 +1650,31 @@
         <v>18</v>
       </c>
       <c r="C5" s="14">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G5" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="H5" s="13">
-        <v>5</v>
+      <c r="H5" s="13" t="s">
+        <v>25</v>
       </c>
       <c r="I5" s="13">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J5" s="13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>17</v>
       </c>
@@ -1665,28 +1682,31 @@
         <v>18</v>
       </c>
       <c r="C6" s="14">
-        <v>46276</v>
+        <v>46277</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>25</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G6" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="13">
+      <c r="H6" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="13">
         <v>20</v>
       </c>
-      <c r="I6" s="13">
+      <c r="J6" s="13">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>17</v>
       </c>
@@ -1694,13 +1714,13 @@
         <v>18</v>
       </c>
       <c r="C7" s="14">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F7" s="13" t="s">
         <v>24</v>
@@ -1708,14 +1728,17 @@
       <c r="G7" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="13">
         <v>46</v>
       </c>
-      <c r="I7" s="13">
+      <c r="J7" s="13">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
         <v>26</v>
       </c>
@@ -1723,26 +1746,29 @@
         <v>27</v>
       </c>
       <c r="C8" s="19">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E8" s="18" t="s">
         <v>25</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G8" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="H8" s="18">
+      <c r="H8" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="I8" s="18">
         <v>0</v>
       </c>
-      <c r="I8" s="18"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J8" s="18"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
         <v>26</v>
       </c>
@@ -1750,28 +1776,31 @@
         <v>27</v>
       </c>
       <c r="C9" s="19">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G9" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="18">
-        <v>5</v>
+      <c r="H9" s="18" t="s">
+        <v>29</v>
       </c>
       <c r="I9" s="18">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J9" s="18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
         <v>26</v>
       </c>
@@ -1779,28 +1808,31 @@
         <v>27</v>
       </c>
       <c r="C10" s="19">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>82</v>
-      </c>
-      <c r="H10" s="18">
+        <v>83</v>
+      </c>
+      <c r="H10" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="I10" s="18">
         <v>14</v>
       </c>
-      <c r="I10" s="18">
+      <c r="J10" s="18">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
         <v>26</v>
       </c>
@@ -1808,28 +1840,31 @@
         <v>27</v>
       </c>
       <c r="C11" s="19">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="H11" s="18">
-        <v>25</v>
+        <v>85</v>
+      </c>
+      <c r="H11" s="18" t="s">
+        <v>29</v>
       </c>
       <c r="I11" s="18">
+        <v>25</v>
+      </c>
+      <c r="J11" s="18">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
         <v>26</v>
       </c>
@@ -1837,13 +1872,13 @@
         <v>27</v>
       </c>
       <c r="C12" s="19">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F12" s="18" t="s">
         <v>32</v>
@@ -1851,14 +1886,17 @@
       <c r="G12" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="18">
+      <c r="H12" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="I12" s="18">
         <v>34</v>
       </c>
-      <c r="I12" s="18">
+      <c r="J12" s="18">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>33</v>
       </c>
@@ -1866,10 +1904,10 @@
         <v>34</v>
       </c>
       <c r="C13" s="14">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E13" s="13" t="s">
         <v>25</v>
@@ -1880,12 +1918,15 @@
       <c r="G13" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="H13" s="13">
+      <c r="H13" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I13" s="13">
         <v>0</v>
       </c>
-      <c r="I13" s="13"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J13" s="13"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
         <v>41</v>
       </c>
@@ -1893,10 +1934,10 @@
         <v>42</v>
       </c>
       <c r="C14" s="19">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E14" s="18" t="s">
         <v>25</v>
@@ -1907,12 +1948,15 @@
       <c r="G14" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="H14" s="18">
+      <c r="H14" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="I14" s="18">
         <v>0</v>
       </c>
-      <c r="I14" s="18"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J14" s="18"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>41</v>
       </c>
@@ -1920,28 +1964,31 @@
         <v>42</v>
       </c>
       <c r="C15" s="19">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G15" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="H15" s="18">
-        <v>3</v>
+      <c r="H15" s="18" t="s">
+        <v>25</v>
       </c>
       <c r="I15" s="18">
         <v>3</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J15" s="18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
         <v>41</v>
       </c>
@@ -1949,28 +1996,31 @@
         <v>42</v>
       </c>
       <c r="C16" s="19">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="H16" s="18">
+        <v>45</v>
+      </c>
+      <c r="H16" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="I16" s="18">
         <v>10</v>
       </c>
-      <c r="I16" s="18">
+      <c r="J16" s="18">
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
         <v>41</v>
       </c>
@@ -1978,28 +2028,31 @@
         <v>42</v>
       </c>
       <c r="C17" s="19">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G17" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="H17" s="18">
+      <c r="H17" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="I17" s="18">
         <v>27</v>
       </c>
-      <c r="I17" s="18">
+      <c r="J17" s="18">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
         <v>41</v>
       </c>
@@ -2007,28 +2060,31 @@
         <v>42</v>
       </c>
       <c r="C18" s="19">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G18" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="H18" s="18">
+      <c r="H18" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="I18" s="18">
         <v>40</v>
       </c>
-      <c r="I18" s="18">
+      <c r="J18" s="18">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>41</v>
       </c>
@@ -2036,10 +2092,10 @@
         <v>42</v>
       </c>
       <c r="C19" s="19">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="D19" s="24" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E19" s="18" t="s">
         <v>25</v>
@@ -2050,14 +2106,17 @@
       <c r="G19" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="H19" s="18">
+      <c r="H19" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="I19" s="18">
         <v>48</v>
       </c>
-      <c r="I19" s="18">
+      <c r="J19" s="18">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>49</v>
       </c>
@@ -2065,10 +2124,10 @@
         <v>50</v>
       </c>
       <c r="C20" s="14">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E20" s="13" t="s">
         <v>25</v>
@@ -2079,12 +2138,15 @@
       <c r="G20" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="H20" s="13">
+      <c r="H20" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I20" s="13">
         <v>0</v>
       </c>
-      <c r="I20" s="13"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J20" s="13"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
         <v>49</v>
       </c>
@@ -2092,28 +2154,31 @@
         <v>50</v>
       </c>
       <c r="C21" s="14">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>25</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G21" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="H21" s="13">
-        <v>13</v>
+      <c r="H21" s="13" t="s">
+        <v>25</v>
       </c>
       <c r="I21" s="13">
         <v>13</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J21" s="13">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
         <v>49</v>
       </c>
@@ -2121,10 +2186,10 @@
         <v>50</v>
       </c>
       <c r="C22" s="14">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>25</v>
@@ -2135,14 +2200,17 @@
       <c r="G22" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="H22" s="13">
+      <c r="H22" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I22" s="13">
         <v>39</v>
       </c>
-      <c r="I22" s="13">
+      <c r="J22" s="13">
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
         <v>56</v>
       </c>
@@ -2150,10 +2218,10 @@
         <v>57</v>
       </c>
       <c r="C23" s="19">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E23" s="18" t="s">
         <v>25</v>
@@ -2164,12 +2232,15 @@
       <c r="G23" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="H23" s="18">
+      <c r="H23" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="I23" s="18">
         <v>0</v>
       </c>
-      <c r="I23" s="18"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J23" s="18"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
         <v>56</v>
       </c>
@@ -2177,28 +2248,31 @@
         <v>57</v>
       </c>
       <c r="C24" s="19">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E24" s="18" t="s">
         <v>25</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G24" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="H24" s="18">
-        <v>14</v>
+      <c r="H24" s="18" t="s">
+        <v>25</v>
       </c>
       <c r="I24" s="18">
         <v>14</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J24" s="18">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
         <v>56</v>
       </c>
@@ -2206,10 +2280,10 @@
         <v>57</v>
       </c>
       <c r="C25" s="19">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="D25" s="24" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E25" s="18" t="s">
         <v>25</v>
@@ -2220,18 +2294,21 @@
       <c r="G25" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="H25" s="18">
+      <c r="H25" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="I25" s="18">
         <v>44</v>
       </c>
-      <c r="I25" s="18">
+      <c r="J25" s="18">
         <v>30</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:I3"/>
+  <autoFilter ref="A3:J3"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2250,7 +2327,7 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -2272,7 +2349,7 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -2306,46 +2383,46 @@
         <v>12</v>
       </c>
       <c r="E3" s="28" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G3" s="28" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H3" s="28" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I3" s="28" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="J3" s="28" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K3" s="28" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="L3" s="28" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="M3" s="28" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="N3" s="28" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="O3" s="28" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="P3" s="28" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="Q3" s="28" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="R3" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -2368,17 +2445,17 @@
       <c r="I4" s="32"/>
       <c r="J4" s="32"/>
       <c r="K4" s="33" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L4" s="34"/>
-      <c r="M4" s="33" t="s">
-        <v>110</v>
-      </c>
-      <c r="N4" s="34"/>
+      <c r="M4" s="34"/>
+      <c r="N4" s="33" t="s">
+        <v>112</v>
+      </c>
       <c r="O4" s="34"/>
       <c r="P4" s="34"/>
       <c r="Q4" s="35" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="R4" s="34"/>
     </row>
@@ -2403,20 +2480,20 @@
       <c r="J5" s="32"/>
       <c r="K5" s="32"/>
       <c r="L5" s="36" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="N5" s="33" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="O5" s="34"/>
       <c r="P5" s="33" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="Q5" s="37" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="R5" s="34"/>
     </row>
@@ -2446,7 +2523,7 @@
       <c r="O6" s="32"/>
       <c r="P6" s="32"/>
       <c r="Q6" s="39" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="R6" s="40"/>
     </row>
@@ -2468,24 +2545,24 @@
       <c r="G7" s="32"/>
       <c r="H7" s="32"/>
       <c r="I7" s="42" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J7" s="43" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K7" s="44" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L7" s="45"/>
       <c r="M7" s="46" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="N7" s="45"/>
       <c r="O7" s="43" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="P7" s="47" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="Q7" s="32"/>
       <c r="R7" s="32"/>
@@ -2509,17 +2586,17 @@
       <c r="H8" s="32"/>
       <c r="I8" s="32"/>
       <c r="J8" s="49" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K8" s="50"/>
       <c r="L8" s="51" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="M8" s="50"/>
       <c r="N8" s="50"/>
       <c r="O8" s="50"/>
       <c r="P8" s="52" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="Q8" s="50"/>
       <c r="R8" s="50"/>
@@ -2538,19 +2615,19 @@
         <v>44</v>
       </c>
       <c r="E9" s="42" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F9" s="45"/>
       <c r="G9" s="43" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H9" s="45"/>
       <c r="I9" s="45"/>
       <c r="J9" s="45"/>
-      <c r="K9" s="47" t="s">
-        <v>111</v>
-      </c>
-      <c r="L9" s="32"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="47" t="s">
+        <v>113</v>
+      </c>
       <c r="M9" s="32"/>
       <c r="N9" s="32"/>
       <c r="O9" s="32"/>

</xml_diff>

<commit_message>
V11: letter / minutes / decision number on events
- New optional field 'رقم الخطاب / المحضر / القرار' in the event form
  (before adding to the timeline) and in the closing form; editable,
  searchable, shown as a tag in the app timeline
- Formal report: own column after the tool in the action log (columns
  narrowed so pages keep their length); consulting and modern styles
  show it with the executor/recipient line; Excel has its own column
- Modern step cards cap text lines so the page height stays stable

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vq5DRv9yx8RnT5NY8AHtK
</commit_message>
<xml_diff>
--- a/samples/5-ملف-Excel.xlsx
+++ b/samples/5-ملف-Excel.xlsx
@@ -193,7 +193,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="117">
   <si>
     <t>ملخص المواضيع</t>
   </si>
@@ -390,6 +390,9 @@
     <t>أداة الحدث</t>
   </si>
   <si>
+    <t>رقم الخطاب / المحضر / القرار</t>
+  </si>
+  <si>
     <t>ما تم</t>
   </si>
   <si>
@@ -435,6 +438,9 @@
     <t>خطاب</t>
   </si>
   <si>
+    <t>4471/ت/1448</t>
+  </si>
+  <si>
     <t>إرسال خطاب للجهة بطلب استيفاء متطلبات الدروع وخطة الوقاية الإشعاعية</t>
   </si>
   <si>
@@ -445,6 +451,9 @@
   </si>
   <si>
     <t>فريق التفتيش</t>
+  </si>
+  <si>
+    <t>محضر 12/1448</t>
   </si>
   <si>
     <t>اجتماع مع الجهة لمناقشة خطة معالجة الملاحظات وجدولها الزمني</t>
@@ -1539,20 +1548,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="13" style="1" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="58" customWidth="1"/>
-    <col min="7" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="52" customWidth="1"/>
+    <col min="8" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>61</v>
       </c>
@@ -1565,8 +1575,9 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="2"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1579,8 +1590,9 @@
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1611,8 +1623,11 @@
       <c r="J3" s="4" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>17</v>
       </c>
@@ -1623,26 +1638,29 @@
         <v>46257</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>25</v>
       </c>
       <c r="F4" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="G4" s="13" t="s">
-        <v>25</v>
-      </c>
       <c r="H4" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="I4" s="13">
+      <c r="I4" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" s="13">
         <v>0</v>
       </c>
-      <c r="J4" s="13"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4" s="13"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>17</v>
       </c>
@@ -1653,28 +1671,31 @@
         <v>46262</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="H5" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="13">
-        <v>5</v>
+      <c r="I5" s="13" t="s">
+        <v>25</v>
       </c>
       <c r="J5" s="13">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K5" s="13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>17</v>
       </c>
@@ -1685,28 +1706,31 @@
         <v>46277</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>25</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="H6" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="13">
+      <c r="I6" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="J6" s="13">
         <v>20</v>
       </c>
-      <c r="J6" s="13">
+      <c r="K6" s="13">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>17</v>
       </c>
@@ -1717,28 +1741,31 @@
         <v>46303</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F7" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="13" t="s">
-        <v>25</v>
-      </c>
       <c r="H7" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="I7" s="13">
+      <c r="I7" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7" s="13">
         <v>46</v>
       </c>
-      <c r="J7" s="13">
+      <c r="K7" s="13">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
         <v>26</v>
       </c>
@@ -1749,26 +1776,29 @@
         <v>46267</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E8" s="18" t="s">
         <v>25</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>25</v>
+        <v>78</v>
       </c>
       <c r="H8" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="I8" s="18">
+      <c r="I8" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="J8" s="18">
         <v>0</v>
       </c>
-      <c r="J8" s="18"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K8" s="18"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
         <v>26</v>
       </c>
@@ -1779,28 +1809,31 @@
         <v>46272</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G9" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="H9" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="18" t="s">
+      <c r="I9" s="18" t="s">
         <v>29</v>
-      </c>
-      <c r="I9" s="18">
-        <v>5</v>
       </c>
       <c r="J9" s="18">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K9" s="18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
         <v>26</v>
       </c>
@@ -1811,28 +1844,31 @@
         <v>46281</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>82</v>
+        <v>25</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="I10" s="18">
+        <v>85</v>
+      </c>
+      <c r="I10" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="J10" s="18">
         <v>14</v>
       </c>
-      <c r="J10" s="18">
+      <c r="K10" s="18">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
         <v>26</v>
       </c>
@@ -1843,28 +1879,31 @@
         <v>46292</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H11" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="I11" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="I11" s="18">
-        <v>25</v>
-      </c>
       <c r="J11" s="18">
+        <v>25</v>
+      </c>
+      <c r="K11" s="18">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
         <v>26</v>
       </c>
@@ -1875,28 +1914,31 @@
         <v>46301</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F12" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G12" s="18" t="s">
+      <c r="H12" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="H12" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="I12" s="18">
+      <c r="I12" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="J12" s="18">
         <v>34</v>
       </c>
-      <c r="J12" s="18">
+      <c r="K12" s="18">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>33</v>
       </c>
@@ -1907,26 +1949,29 @@
         <v>46299</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E13" s="13" t="s">
         <v>25</v>
       </c>
       <c r="F13" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="G13" s="13" t="s">
-        <v>25</v>
-      </c>
       <c r="H13" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="I13" s="13">
+      <c r="I13" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="J13" s="13">
         <v>0</v>
       </c>
-      <c r="J13" s="13"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K13" s="13"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
         <v>41</v>
       </c>
@@ -1937,26 +1982,29 @@
         <v>46247</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" s="18" t="s">
         <v>25</v>
       </c>
       <c r="F14" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="G14" s="18" t="s">
-        <v>25</v>
-      </c>
       <c r="H14" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="I14" s="18">
+      <c r="I14" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="J14" s="18">
         <v>0</v>
       </c>
-      <c r="J14" s="18"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K14" s="18"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>41</v>
       </c>
@@ -1967,28 +2015,31 @@
         <v>46250</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>88</v>
+        <v>25</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="H15" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="I15" s="18">
-        <v>3</v>
+      <c r="I15" s="18" t="s">
+        <v>25</v>
       </c>
       <c r="J15" s="18">
         <v>3</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K15" s="18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
         <v>41</v>
       </c>
@@ -1999,28 +2050,31 @@
         <v>46257</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>89</v>
+        <v>25</v>
       </c>
       <c r="G16" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="H16" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="H16" s="18" t="s">
+      <c r="I16" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="I16" s="18">
+      <c r="J16" s="18">
         <v>10</v>
       </c>
-      <c r="J16" s="18">
+      <c r="K16" s="18">
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
         <v>41</v>
       </c>
@@ -2031,28 +2085,31 @@
         <v>46274</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>90</v>
+        <v>25</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="H17" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="I17" s="18">
+      <c r="I17" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="J17" s="18">
         <v>27</v>
       </c>
-      <c r="J17" s="18">
+      <c r="K17" s="18">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
         <v>41</v>
       </c>
@@ -2063,28 +2120,31 @@
         <v>46287</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>25</v>
+        <v>94</v>
       </c>
       <c r="H18" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="I18" s="18">
+      <c r="I18" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="J18" s="18">
         <v>40</v>
       </c>
-      <c r="J18" s="18">
+      <c r="K18" s="18">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>41</v>
       </c>
@@ -2095,28 +2155,31 @@
         <v>46295</v>
       </c>
       <c r="D19" s="24" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E19" s="18" t="s">
         <v>25</v>
       </c>
       <c r="F19" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="G19" s="18" t="s">
-        <v>25</v>
-      </c>
       <c r="H19" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="I19" s="18">
+      <c r="I19" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="J19" s="18">
         <v>48</v>
       </c>
-      <c r="J19" s="18">
+      <c r="K19" s="18">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>49</v>
       </c>
@@ -2127,26 +2190,29 @@
         <v>46255</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E20" s="13" t="s">
         <v>25</v>
       </c>
       <c r="F20" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="G20" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="G20" s="13" t="s">
-        <v>25</v>
-      </c>
       <c r="H20" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="I20" s="13">
+      <c r="I20" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="J20" s="13">
         <v>0</v>
       </c>
-      <c r="J20" s="13"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K20" s="13"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
         <v>49</v>
       </c>
@@ -2157,28 +2223,31 @@
         <v>46268</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>25</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="H21" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="I21" s="13">
-        <v>13</v>
+      <c r="I21" s="13" t="s">
+        <v>25</v>
       </c>
       <c r="J21" s="13">
         <v>13</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K21" s="13">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
         <v>49</v>
       </c>
@@ -2189,28 +2258,31 @@
         <v>46294</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>25</v>
       </c>
       <c r="F22" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="G22" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="G22" s="13" t="s">
-        <v>25</v>
-      </c>
       <c r="H22" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="I22" s="13">
+      <c r="I22" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="J22" s="13">
         <v>39</v>
       </c>
-      <c r="J22" s="13">
+      <c r="K22" s="13">
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
         <v>56</v>
       </c>
@@ -2221,26 +2293,29 @@
         <v>46219</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E23" s="18" t="s">
         <v>25</v>
       </c>
       <c r="F23" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G23" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="G23" s="18" t="s">
-        <v>25</v>
-      </c>
       <c r="H23" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="I23" s="18">
+      <c r="I23" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="J23" s="18">
         <v>0</v>
       </c>
-      <c r="J23" s="18"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K23" s="18"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
         <v>56</v>
       </c>
@@ -2251,28 +2326,31 @@
         <v>46233</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E24" s="18" t="s">
         <v>25</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>94</v>
+        <v>25</v>
       </c>
       <c r="G24" s="18" t="s">
-        <v>25</v>
+        <v>97</v>
       </c>
       <c r="H24" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="I24" s="18">
-        <v>14</v>
+      <c r="I24" s="18" t="s">
+        <v>25</v>
       </c>
       <c r="J24" s="18">
         <v>14</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K24" s="18">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
         <v>56</v>
       </c>
@@ -2283,32 +2361,35 @@
         <v>46263</v>
       </c>
       <c r="D25" s="24" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E25" s="18" t="s">
         <v>25</v>
       </c>
       <c r="F25" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G25" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="G25" s="18" t="s">
-        <v>25</v>
-      </c>
       <c r="H25" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="I25" s="18">
+      <c r="I25" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="J25" s="18">
         <v>44</v>
       </c>
-      <c r="J25" s="18">
+      <c r="K25" s="18">
         <v>30</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J3"/>
+  <autoFilter ref="A3:K3"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2327,7 +2408,7 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -2349,7 +2430,7 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -2383,46 +2464,46 @@
         <v>12</v>
       </c>
       <c r="E3" s="28" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G3" s="28" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H3" s="28" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="I3" s="28" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="J3" s="28" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="K3" s="28" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="L3" s="28" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="M3" s="28" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="N3" s="28" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="O3" s="28" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="P3" s="28" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="Q3" s="28" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="R3" s="29" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -2445,17 +2526,17 @@
       <c r="I4" s="32"/>
       <c r="J4" s="32"/>
       <c r="K4" s="33" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="L4" s="34"/>
       <c r="M4" s="34"/>
       <c r="N4" s="33" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="O4" s="34"/>
       <c r="P4" s="34"/>
       <c r="Q4" s="35" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="R4" s="34"/>
     </row>
@@ -2480,20 +2561,20 @@
       <c r="J5" s="32"/>
       <c r="K5" s="32"/>
       <c r="L5" s="36" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="N5" s="33" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="O5" s="34"/>
       <c r="P5" s="33" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="Q5" s="37" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="R5" s="34"/>
     </row>
@@ -2523,7 +2604,7 @@
       <c r="O6" s="32"/>
       <c r="P6" s="32"/>
       <c r="Q6" s="39" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="R6" s="40"/>
     </row>
@@ -2545,24 +2626,24 @@
       <c r="G7" s="32"/>
       <c r="H7" s="32"/>
       <c r="I7" s="42" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="J7" s="43" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K7" s="44" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="L7" s="45"/>
       <c r="M7" s="46" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="N7" s="45"/>
       <c r="O7" s="43" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="P7" s="47" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="Q7" s="32"/>
       <c r="R7" s="32"/>
@@ -2586,17 +2667,17 @@
       <c r="H8" s="32"/>
       <c r="I8" s="32"/>
       <c r="J8" s="49" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K8" s="50"/>
       <c r="L8" s="51" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="M8" s="50"/>
       <c r="N8" s="50"/>
       <c r="O8" s="50"/>
       <c r="P8" s="52" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="Q8" s="50"/>
       <c r="R8" s="50"/>
@@ -2615,18 +2696,18 @@
         <v>44</v>
       </c>
       <c r="E9" s="42" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F9" s="45"/>
       <c r="G9" s="43" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="H9" s="45"/>
       <c r="I9" s="45"/>
       <c r="J9" s="45"/>
       <c r="K9" s="45"/>
       <c r="L9" s="47" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="M9" s="32"/>
       <c r="N9" s="32"/>

</xml_diff>

<commit_message>
V13: Hijri dates, automatic backups and an audit log
- Calendar setting (Gregorian + Hijri / Gregorian / Hijri, Umm al-Qura) applied
  to the app, the three report styles, date-field hints and a Hijri column in Excel
- Shared mode: daily backup to backups/backup-YYYY-MM-DD.json in the shared
  folder, newest 30 kept; local mode: reminder after 7 days without a backup
- Audit log per topic (field changes, event add/edit/delete, who and when)
  merged across devices, plus a deleted-topics list; shown in the app only
- Fix: deleting an event while a background sync replaced the data was lost;
  guard edits of topics/events deleted on another device

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vq5DRv9yx8RnT5NY8AHtK
</commit_message>
<xml_diff>
--- a/samples/5-ملف-Excel.xlsx
+++ b/samples/5-ملف-Excel.xlsx
@@ -21,9 +21,9 @@
     <comment ref="K4" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/23 – فتح الموضوع
+          <t xml:space="preserve">2026/08/23م – 1448/03/10هـ – فتح الموضوع
 تسجيل الموضوع
-2026/08/28 – إجراء · اجتماع
+2026/08/28م – 1448/03/15هـ – إجراء · اجتماع
 ورشة عمل داخلية لمراجعة المسودة الأولى</t>
         </r>
       </text>
@@ -31,7 +31,7 @@
     <comment ref="N4" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/12 – إجراء
+          <t xml:space="preserve">2026/09/12م – 1448/04/01هـ – إجراء
 طرح المسودة لأخذ مرئيات الجهات ذات العلاقة</t>
         </r>
       </text>
@@ -39,7 +39,7 @@
     <comment ref="Q4" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/10/08 – تحديث · بريد إلكتروني
+          <t xml:space="preserve">2026/10/08م – 1448/04/27هـ – تحديث · بريد إلكتروني
 استلام 12 مرئية من الجهات</t>
         </r>
       </text>
@@ -47,7 +47,7 @@
     <comment ref="L5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/02 – فتح الموضوع
+          <t xml:space="preserve">2026/09/02م – 1448/03/20هـ – فتح الموضوع
 تسجيل الموضوع: طلب ترخيص جديد لاستخدام مصادر مشعة في العلاج الإشعاعي، ويتطلب استيفاء متطلبات الدروع والتقييم الإشعاعي قبل إصدار الترخيص.</t>
         </r>
       </text>
@@ -55,7 +55,7 @@
     <comment ref="M5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/07 – متابعة · خطاب – المنفذ: أحمد العتيبي – المستلم: جهة طبية طالبة للترخيص
+          <t xml:space="preserve">2026/09/07م – 1448/03/25هـ – متابعة · خطاب – المنفذ: أحمد العتيبي – المستلم: جهة طبية طالبة للترخيص
 إرسال خطاب للجهة بطلب استيفاء متطلبات الدروع وخطة الوقاية الإشعاعية</t>
         </r>
       </text>
@@ -63,7 +63,7 @@
     <comment ref="N5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/16 – إجراء · زيارة ميدانية – المنفذ: فريق التفتيش
+          <t xml:space="preserve">2026/09/16م – 1448/04/05هـ – إجراء · زيارة ميدانية – المنفذ: فريق التفتيش
 زيارة ميدانية للتحقق من غرفة العلاج وأنظمة الدروع؛ رُصدت 3 ملاحظات</t>
         </r>
       </text>
@@ -71,7 +71,7 @@
     <comment ref="P5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/27 – إجراء · اجتماع – المنفذ: إدارة التراخيص – المستلم: جهة طبية طالبة للترخيص
+          <t xml:space="preserve">2026/09/27م – 1448/04/16هـ – إجراء · اجتماع – المنفذ: إدارة التراخيص – المستلم: جهة طبية طالبة للترخيص
 اجتماع مع الجهة لمناقشة خطة معالجة الملاحظات وجدولها الزمني</t>
         </r>
       </text>
@@ -79,7 +79,7 @@
     <comment ref="Q5" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/10/06 – متابعة · اتصال هاتفي – المنفذ: أحمد العتيبي – المستلم: مسؤول الوقاية الإشعاعية بالجهة
+          <t xml:space="preserve">2026/10/06م – 1448/04/25هـ – متابعة · اتصال هاتفي – المنفذ: أحمد العتيبي – المستلم: مسؤول الوقاية الإشعاعية بالجهة
 متابعة تنفيذ تعديلات الدروع – بانتظار تقرير القياس من الجهة</t>
         </r>
       </text>
@@ -87,7 +87,7 @@
     <comment ref="Q6" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/10/04 – فتح الموضوع
+          <t xml:space="preserve">2026/10/04م – 1448/04/23هـ – فتح الموضوع
 تسجيل الموضوع</t>
         </r>
       </text>
@@ -95,7 +95,7 @@
     <comment ref="I7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/13 – فتح الموضوع
+          <t xml:space="preserve">2026/08/13م – 1448/02/30هـ – فتح الموضوع
 تسجيل الموضوع</t>
         </r>
       </text>
@@ -103,7 +103,7 @@
     <comment ref="J7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/16 – إجراء · زيارة ميدانية
+          <t xml:space="preserve">2026/08/16م – 1448/03/03هـ – إجراء · زيارة ميدانية
 تفتيش دوري ورصد 5 ملاحظات على حفظ المصادر وسجلات الجرعات</t>
         </r>
       </text>
@@ -111,7 +111,7 @@
     <comment ref="K7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/23 – متابعة · خطاب – المنفذ: سارة القحطاني – المستلم: منشأة صناعية مرخَّص لها
+          <t xml:space="preserve">2026/08/23م – 1448/03/10هـ – متابعة · خطاب – المنفذ: سارة القحطاني – المستلم: منشأة صناعية مرخَّص لها
 إبلاغ المنشأة بالملاحظات ومهلة المعالجة</t>
         </r>
       </text>
@@ -119,7 +119,7 @@
     <comment ref="M7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/09 – تحديث · بريد إلكتروني
+          <t xml:space="preserve">2026/09/09م – 1448/03/27هـ – تحديث · بريد إلكتروني
 استلام شواهد معالجة 4 ملاحظات</t>
         </r>
       </text>
@@ -127,7 +127,7 @@
     <comment ref="O7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/22 – إجراء · زيارة ميدانية
+          <t xml:space="preserve">2026/09/22م – 1448/04/11هـ – إجراء · زيارة ميدانية
 زيارة تحقق ميدانية من المعالجة</t>
         </r>
       </text>
@@ -135,7 +135,7 @@
     <comment ref="P7" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/30 – إقفال
+          <t xml:space="preserve">2026/09/30م – 1448/04/19هـ – إقفال
 التحقق من معالجة جميع الملاحظات وإغلاقها</t>
         </r>
       </text>
@@ -143,7 +143,7 @@
     <comment ref="J8" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/21 – فتح الموضوع
+          <t xml:space="preserve">2026/08/21م – 1448/03/08هـ – فتح الموضوع
 تسجيل الموضوع</t>
         </r>
       </text>
@@ -151,7 +151,7 @@
     <comment ref="L8" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/03 – إجراء
+          <t xml:space="preserve">2026/09/03م – 1448/03/21هـ – إجراء
 إعداد سيناريو التمرين وخطة التقييم</t>
         </r>
       </text>
@@ -159,7 +159,7 @@
     <comment ref="P8" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/09/29 – متابعة
+          <t xml:space="preserve">2026/09/29م – 1448/04/18هـ – متابعة
 تعليق موعد التمرين بانتظار تأكيد الجهات المشاركة</t>
         </r>
       </text>
@@ -167,7 +167,7 @@
     <comment ref="E9" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/07/16 – فتح الموضوع
+          <t xml:space="preserve">2026/07/16م – 1448/02/02هـ – فتح الموضوع
 تسجيل الموضوع</t>
         </r>
       </text>
@@ -175,7 +175,7 @@
     <comment ref="G9" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/07/30 – إجراء
+          <t xml:space="preserve">2026/07/30م – 1448/02/16هـ – إجراء
 حصر المصادر لدى الجهات المرخَّص لها ومطابقتها مع السجل</t>
         </r>
       </text>
@@ -183,7 +183,7 @@
     <comment ref="L9" authorId="0">
       <text>
         <r>
-          <t xml:space="preserve">2026/08/29 – إقفال
+          <t xml:space="preserve">2026/08/29م – 1448/03/16هـ – إقفال
 اعتماد السجل المحدّث ونشره داخلياً</t>
         </r>
       </text>
@@ -193,12 +193,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="139">
   <si>
     <t>ملخص المواضيع</t>
   </si>
   <si>
-    <t>تاريخ الإصدار: 2026/10/12</t>
+    <t>تاريخ الإصدار: 2026/10/12م – 1448/05/01هـ</t>
   </si>
   <si>
     <t>المرجع</t>
@@ -384,6 +384,9 @@
     <t>التاريخ</t>
   </si>
   <si>
+    <t>التاريخ الهجري</t>
+  </si>
+  <si>
     <t>نوع الحدث</t>
   </si>
   <si>
@@ -408,9 +411,15 @@
     <t>الفاصل عن الحدث السابق (يوم)</t>
   </si>
   <si>
+    <t>1448/03/10</t>
+  </si>
+  <si>
     <t>فتح الموضوع</t>
   </si>
   <si>
+    <t>1448/03/15</t>
+  </si>
+  <si>
     <t>إجراء</t>
   </si>
   <si>
@@ -420,18 +429,30 @@
     <t>ورشة عمل داخلية لمراجعة المسودة الأولى</t>
   </si>
   <si>
+    <t>1448/04/01</t>
+  </si>
+  <si>
     <t>طرح المسودة لأخذ مرئيات الجهات ذات العلاقة</t>
   </si>
   <si>
+    <t>1448/04/27</t>
+  </si>
+  <si>
     <t>تحديث</t>
   </si>
   <si>
     <t>بريد إلكتروني</t>
   </si>
   <si>
+    <t>1448/03/20</t>
+  </si>
+  <si>
     <t>تسجيل الموضوع: طلب ترخيص جديد لاستخدام مصادر مشعة في العلاج الإشعاعي، ويتطلب استيفاء متطلبات الدروع والتقييم الإشعاعي قبل إصدار الترخيص.</t>
   </si>
   <si>
+    <t>1448/03/25</t>
+  </si>
+  <si>
     <t>متابعة</t>
   </si>
   <si>
@@ -444,6 +465,9 @@
     <t>إرسال خطاب للجهة بطلب استيفاء متطلبات الدروع وخطة الوقاية الإشعاعية</t>
   </si>
   <si>
+    <t>1448/04/05</t>
+  </si>
+  <si>
     <t>زيارة ميدانية</t>
   </si>
   <si>
@@ -453,6 +477,9 @@
     <t>فريق التفتيش</t>
   </si>
   <si>
+    <t>1448/04/16</t>
+  </si>
+  <si>
     <t>محضر 12/1448</t>
   </si>
   <si>
@@ -462,31 +489,70 @@
     <t>إدارة التراخيص</t>
   </si>
   <si>
+    <t>1448/04/25</t>
+  </si>
+  <si>
     <t>اتصال هاتفي</t>
   </si>
   <si>
     <t>مسؤول الوقاية الإشعاعية بالجهة</t>
   </si>
   <si>
+    <t>1448/04/23</t>
+  </si>
+  <si>
+    <t>1448/02/30</t>
+  </si>
+  <si>
+    <t>1448/03/03</t>
+  </si>
+  <si>
     <t>تفتيش دوري ورصد 5 ملاحظات على حفظ المصادر وسجلات الجرعات</t>
   </si>
   <si>
     <t>إبلاغ المنشأة بالملاحظات ومهلة المعالجة</t>
   </si>
   <si>
+    <t>1448/03/27</t>
+  </si>
+  <si>
     <t>استلام شواهد معالجة 4 ملاحظات</t>
   </si>
   <si>
+    <t>1448/04/11</t>
+  </si>
+  <si>
     <t>زيارة تحقق ميدانية من المعالجة</t>
   </si>
   <si>
+    <t>1448/04/19</t>
+  </si>
+  <si>
     <t>إقفال</t>
   </si>
   <si>
+    <t>1448/03/08</t>
+  </si>
+  <si>
+    <t>1448/03/21</t>
+  </si>
+  <si>
     <t>إعداد سيناريو التمرين وخطة التقييم</t>
   </si>
   <si>
+    <t>1448/04/18</t>
+  </si>
+  <si>
+    <t>1448/02/02</t>
+  </si>
+  <si>
+    <t>1448/02/16</t>
+  </si>
+  <si>
     <t>حصر المصادر لدى الجهات المرخَّص لها ومطابقتها مع السجل</t>
+  </si>
+  <si>
+    <t>1448/03/16</t>
   </si>
   <si>
     <t>المخطط الزمني (Timeline) – عرض أسبوعي (يبدأ السبت)</t>
@@ -1548,21 +1614,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="13" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="52" customWidth="1"/>
-    <col min="8" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="52" customWidth="1"/>
+    <col min="9" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>61</v>
       </c>
@@ -1576,8 +1643,9 @@
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" s="2"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1591,8 +1659,9 @@
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2" s="3"/>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1626,8 +1695,11 @@
       <c r="K3" s="4" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>17</v>
       </c>
@@ -1637,30 +1709,33 @@
       <c r="C4" s="14">
         <v>46257</v>
       </c>
-      <c r="D4" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>25</v>
+      <c r="D4" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="F4" s="13" t="s">
         <v>25</v>
       </c>
       <c r="G4" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="H4" s="13" t="s">
-        <v>25</v>
-      </c>
       <c r="I4" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="13">
+      <c r="J4" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="K4" s="13">
         <v>0</v>
       </c>
-      <c r="K4" s="13"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4" s="13"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>17</v>
       </c>
@@ -1670,32 +1745,35 @@
       <c r="C5" s="14">
         <v>46262</v>
       </c>
-      <c r="D5" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>73</v>
+      <c r="D5" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>75</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>25</v>
+        <v>77</v>
       </c>
       <c r="I5" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J5" s="13">
-        <v>5</v>
+      <c r="J5" s="13" t="s">
+        <v>25</v>
       </c>
       <c r="K5" s="13">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5" s="13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>17</v>
       </c>
@@ -1705,32 +1783,35 @@
       <c r="C6" s="14">
         <v>46277</v>
       </c>
-      <c r="D6" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>25</v>
+      <c r="D6" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>75</v>
       </c>
       <c r="F6" s="13" t="s">
         <v>25</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>25</v>
+        <v>79</v>
       </c>
       <c r="I6" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J6" s="13">
+      <c r="J6" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="K6" s="13">
         <v>20</v>
       </c>
-      <c r="K6" s="13">
+      <c r="L6" s="13">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>17</v>
       </c>
@@ -1740,32 +1821,35 @@
       <c r="C7" s="14">
         <v>46303</v>
       </c>
-      <c r="D7" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>77</v>
+      <c r="D7" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>81</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>25</v>
+        <v>82</v>
       </c>
       <c r="G7" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="H7" s="13" t="s">
-        <v>25</v>
-      </c>
       <c r="I7" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J7" s="13">
+      <c r="J7" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="K7" s="13">
         <v>46</v>
       </c>
-      <c r="K7" s="13">
+      <c r="L7" s="13">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
         <v>26</v>
       </c>
@@ -1775,30 +1859,33 @@
       <c r="C8" s="19">
         <v>46267</v>
       </c>
-      <c r="D8" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>25</v>
+      <c r="D8" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" s="20" t="s">
+        <v>73</v>
       </c>
       <c r="F8" s="18" t="s">
         <v>25</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="I8" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="J8" s="18">
+      <c r="J8" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="K8" s="18">
         <v>0</v>
       </c>
-      <c r="K8" s="18"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L8" s="18"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
         <v>26</v>
       </c>
@@ -1808,32 +1895,35 @@
       <c r="C9" s="19">
         <v>46272</v>
       </c>
-      <c r="D9" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>80</v>
+      <c r="D9" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>86</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="H9" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="I9" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I9" s="18" t="s">
+      <c r="J9" s="18" t="s">
         <v>29</v>
-      </c>
-      <c r="J9" s="18">
-        <v>5</v>
       </c>
       <c r="K9" s="18">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L9" s="18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
         <v>26</v>
       </c>
@@ -1843,32 +1933,35 @@
       <c r="C10" s="19">
         <v>46281</v>
       </c>
-      <c r="D10" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>83</v>
+      <c r="D10" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>75</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>84</v>
+        <v>25</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="I10" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="J10" s="18">
+        <v>93</v>
+      </c>
+      <c r="J10" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="K10" s="18">
         <v>14</v>
       </c>
-      <c r="K10" s="18">
+      <c r="L10" s="18">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
         <v>26</v>
       </c>
@@ -1878,32 +1971,35 @@
       <c r="C11" s="19">
         <v>46292</v>
       </c>
-      <c r="D11" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>73</v>
+      <c r="D11" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>75</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="H11" s="18" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="I11" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="J11" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="J11" s="18">
-        <v>25</v>
-      </c>
       <c r="K11" s="18">
+        <v>25</v>
+      </c>
+      <c r="L11" s="18">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
         <v>26</v>
       </c>
@@ -1913,32 +2009,35 @@
       <c r="C12" s="19">
         <v>46301</v>
       </c>
-      <c r="D12" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>89</v>
+      <c r="D12" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>86</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>25</v>
+        <v>99</v>
       </c>
       <c r="G12" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="H12" s="18" t="s">
+      <c r="I12" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I12" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="J12" s="18">
+      <c r="J12" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="K12" s="18">
         <v>34</v>
       </c>
-      <c r="K12" s="18">
+      <c r="L12" s="18">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>33</v>
       </c>
@@ -1948,30 +2047,33 @@
       <c r="C13" s="14">
         <v>46299</v>
       </c>
-      <c r="D13" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>25</v>
+      <c r="D13" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>25</v>
       </c>
       <c r="G13" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="H13" s="13" t="s">
-        <v>25</v>
-      </c>
       <c r="I13" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J13" s="13">
+      <c r="J13" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="K13" s="13">
         <v>0</v>
       </c>
-      <c r="K13" s="13"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L13" s="13"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
         <v>41</v>
       </c>
@@ -1981,30 +2083,33 @@
       <c r="C14" s="19">
         <v>46247</v>
       </c>
-      <c r="D14" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>25</v>
+      <c r="D14" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>73</v>
       </c>
       <c r="F14" s="18" t="s">
         <v>25</v>
       </c>
       <c r="G14" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H14" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="H14" s="18" t="s">
-        <v>25</v>
-      </c>
       <c r="I14" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="J14" s="18">
+      <c r="J14" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="K14" s="18">
         <v>0</v>
       </c>
-      <c r="K14" s="18"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L14" s="18"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="18" t="s">
         <v>41</v>
       </c>
@@ -2014,32 +2119,35 @@
       <c r="C15" s="19">
         <v>46250</v>
       </c>
-      <c r="D15" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="E15" s="18" t="s">
-        <v>83</v>
+      <c r="D15" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>75</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="G15" s="18" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="I15" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="J15" s="18">
-        <v>3</v>
+      <c r="J15" s="18" t="s">
+        <v>25</v>
       </c>
       <c r="K15" s="18">
         <v>3</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L15" s="18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
         <v>41</v>
       </c>
@@ -2049,32 +2157,35 @@
       <c r="C16" s="19">
         <v>46257</v>
       </c>
-      <c r="D16" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="E16" s="18" t="s">
-        <v>80</v>
+      <c r="D16" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>86</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>25</v>
+        <v>87</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>92</v>
+        <v>25</v>
       </c>
       <c r="H16" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="I16" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="I16" s="18" t="s">
+      <c r="J16" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="J16" s="18">
+      <c r="K16" s="18">
         <v>10</v>
       </c>
-      <c r="K16" s="18">
+      <c r="L16" s="18">
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
         <v>41</v>
       </c>
@@ -2084,32 +2195,35 @@
       <c r="C17" s="19">
         <v>46274</v>
       </c>
-      <c r="D17" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="E17" s="18" t="s">
-        <v>77</v>
+      <c r="D17" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>81</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>25</v>
+        <v>82</v>
       </c>
       <c r="G17" s="18" t="s">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="H17" s="18" t="s">
-        <v>25</v>
+        <v>107</v>
       </c>
       <c r="I17" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="J17" s="18">
+      <c r="J17" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="K17" s="18">
         <v>27</v>
       </c>
-      <c r="K17" s="18">
+      <c r="L17" s="18">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
         <v>41</v>
       </c>
@@ -2119,32 +2233,35 @@
       <c r="C18" s="19">
         <v>46287</v>
       </c>
-      <c r="D18" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="E18" s="18" t="s">
-        <v>83</v>
+      <c r="D18" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>75</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>94</v>
+        <v>25</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>25</v>
+        <v>109</v>
       </c>
       <c r="I18" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="J18" s="18">
+      <c r="J18" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="K18" s="18">
         <v>40</v>
       </c>
-      <c r="K18" s="18">
+      <c r="L18" s="18">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="18" t="s">
         <v>41</v>
       </c>
@@ -2154,32 +2271,35 @@
       <c r="C19" s="19">
         <v>46295</v>
       </c>
-      <c r="D19" s="24" t="s">
-        <v>95</v>
-      </c>
-      <c r="E19" s="18" t="s">
-        <v>25</v>
+      <c r="D19" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>111</v>
       </c>
       <c r="F19" s="18" t="s">
         <v>25</v>
       </c>
       <c r="G19" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H19" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="H19" s="18" t="s">
-        <v>25</v>
-      </c>
       <c r="I19" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="J19" s="18">
+      <c r="J19" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="K19" s="18">
         <v>48</v>
       </c>
-      <c r="K19" s="18">
+      <c r="L19" s="18">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>49</v>
       </c>
@@ -2189,30 +2309,33 @@
       <c r="C20" s="14">
         <v>46255</v>
       </c>
-      <c r="D20" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>25</v>
+      <c r="D20" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="F20" s="13" t="s">
         <v>25</v>
       </c>
       <c r="G20" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H20" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="H20" s="13" t="s">
-        <v>25</v>
-      </c>
       <c r="I20" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J20" s="13">
+      <c r="J20" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="K20" s="13">
         <v>0</v>
       </c>
-      <c r="K20" s="13"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L20" s="13"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
         <v>49</v>
       </c>
@@ -2222,32 +2345,35 @@
       <c r="C21" s="14">
         <v>46268</v>
       </c>
-      <c r="D21" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>25</v>
+      <c r="D21" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>75</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>25</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>96</v>
+        <v>25</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>25</v>
+        <v>114</v>
       </c>
       <c r="I21" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J21" s="13">
-        <v>13</v>
+      <c r="J21" s="13" t="s">
+        <v>25</v>
       </c>
       <c r="K21" s="13">
         <v>13</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L21" s="13">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
         <v>49</v>
       </c>
@@ -2257,32 +2383,35 @@
       <c r="C22" s="14">
         <v>46294</v>
       </c>
-      <c r="D22" s="25" t="s">
-        <v>79</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>25</v>
+      <c r="D22" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="E22" s="25" t="s">
+        <v>86</v>
       </c>
       <c r="F22" s="13" t="s">
         <v>25</v>
       </c>
       <c r="G22" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H22" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="H22" s="13" t="s">
-        <v>25</v>
-      </c>
       <c r="I22" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J22" s="13">
+      <c r="J22" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="K22" s="13">
         <v>39</v>
       </c>
-      <c r="K22" s="13">
+      <c r="L22" s="13">
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
         <v>56</v>
       </c>
@@ -2292,30 +2421,33 @@
       <c r="C23" s="19">
         <v>46219</v>
       </c>
-      <c r="D23" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>25</v>
+      <c r="D23" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="E23" s="20" t="s">
+        <v>73</v>
       </c>
       <c r="F23" s="18" t="s">
         <v>25</v>
       </c>
       <c r="G23" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H23" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="H23" s="18" t="s">
-        <v>25</v>
-      </c>
       <c r="I23" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="J23" s="18">
+      <c r="J23" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="K23" s="18">
         <v>0</v>
       </c>
-      <c r="K23" s="18"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L23" s="18"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
         <v>56</v>
       </c>
@@ -2325,32 +2457,35 @@
       <c r="C24" s="19">
         <v>46233</v>
       </c>
-      <c r="D24" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="E24" s="18" t="s">
-        <v>25</v>
+      <c r="D24" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="E24" s="22" t="s">
+        <v>75</v>
       </c>
       <c r="F24" s="18" t="s">
         <v>25</v>
       </c>
       <c r="G24" s="18" t="s">
-        <v>97</v>
+        <v>25</v>
       </c>
       <c r="H24" s="18" t="s">
-        <v>25</v>
+        <v>118</v>
       </c>
       <c r="I24" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="J24" s="18">
-        <v>14</v>
+      <c r="J24" s="18" t="s">
+        <v>25</v>
       </c>
       <c r="K24" s="18">
         <v>14</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L24" s="18">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
         <v>56</v>
       </c>
@@ -2360,36 +2495,39 @@
       <c r="C25" s="19">
         <v>46263</v>
       </c>
-      <c r="D25" s="24" t="s">
-        <v>95</v>
-      </c>
-      <c r="E25" s="18" t="s">
-        <v>25</v>
+      <c r="D25" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="E25" s="24" t="s">
+        <v>111</v>
       </c>
       <c r="F25" s="18" t="s">
         <v>25</v>
       </c>
       <c r="G25" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H25" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="H25" s="18" t="s">
-        <v>25</v>
-      </c>
       <c r="I25" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="J25" s="18">
+      <c r="J25" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="K25" s="18">
         <v>44</v>
       </c>
-      <c r="K25" s="18">
+      <c r="L25" s="18">
         <v>30</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:K3"/>
+  <autoFilter ref="A3:L3"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2408,7 +2546,7 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -2430,7 +2568,7 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -2464,46 +2602,46 @@
         <v>12</v>
       </c>
       <c r="E3" s="28" t="s">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
       <c r="G3" s="28" t="s">
-        <v>102</v>
+        <v>124</v>
       </c>
       <c r="H3" s="28" t="s">
-        <v>103</v>
+        <v>125</v>
       </c>
       <c r="I3" s="28" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="J3" s="28" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="K3" s="28" t="s">
-        <v>106</v>
+        <v>128</v>
       </c>
       <c r="L3" s="28" t="s">
-        <v>107</v>
+        <v>129</v>
       </c>
       <c r="M3" s="28" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="N3" s="28" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="O3" s="28" t="s">
-        <v>110</v>
+        <v>132</v>
       </c>
       <c r="P3" s="28" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="Q3" s="28" t="s">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="R3" s="29" t="s">
-        <v>113</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -2526,17 +2664,17 @@
       <c r="I4" s="32"/>
       <c r="J4" s="32"/>
       <c r="K4" s="33" t="s">
-        <v>114</v>
+        <v>136</v>
       </c>
       <c r="L4" s="34"/>
       <c r="M4" s="34"/>
       <c r="N4" s="33" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="O4" s="34"/>
       <c r="P4" s="34"/>
       <c r="Q4" s="35" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="R4" s="34"/>
     </row>
@@ -2561,20 +2699,20 @@
       <c r="J5" s="32"/>
       <c r="K5" s="32"/>
       <c r="L5" s="36" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="N5" s="33" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="O5" s="34"/>
       <c r="P5" s="33" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="Q5" s="37" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="R5" s="34"/>
     </row>
@@ -2604,7 +2742,7 @@
       <c r="O6" s="32"/>
       <c r="P6" s="32"/>
       <c r="Q6" s="39" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="R6" s="40"/>
     </row>
@@ -2626,24 +2764,24 @@
       <c r="G7" s="32"/>
       <c r="H7" s="32"/>
       <c r="I7" s="42" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="J7" s="43" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="K7" s="44" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="L7" s="45"/>
       <c r="M7" s="46" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="N7" s="45"/>
       <c r="O7" s="43" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="P7" s="47" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="Q7" s="32"/>
       <c r="R7" s="32"/>
@@ -2667,17 +2805,17 @@
       <c r="H8" s="32"/>
       <c r="I8" s="32"/>
       <c r="J8" s="49" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="K8" s="50"/>
       <c r="L8" s="51" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="M8" s="50"/>
       <c r="N8" s="50"/>
       <c r="O8" s="50"/>
       <c r="P8" s="52" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="Q8" s="50"/>
       <c r="R8" s="50"/>
@@ -2696,18 +2834,18 @@
         <v>44</v>
       </c>
       <c r="E9" s="42" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="F9" s="45"/>
       <c r="G9" s="43" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="H9" s="45"/>
       <c r="I9" s="45"/>
       <c r="J9" s="45"/>
       <c r="K9" s="45"/>
       <c r="L9" s="47" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="M9" s="32"/>
       <c r="N9" s="32"/>

</xml_diff>